<commit_message>
data: Hill's Prescription Diet + Science Plan from the April-2026 price-list PDFs
- new positional parser: price | 8-digit SKU | pack size columns + a name cell merged
  across its size rows, matched by nearest baseline; wrapped names joined, gram packs kept
- PD replaces the clinic TS rows — every matched row differed (TS was ~3.5% lower);
  the food indication is carried over from the TS by name+size
- Science Plan (85) is a new retail food list; Vet Essentials stays TS-only and flagged
- Hill's letter codes (c/d k/d i/d j/d l/d t/d y/d z/d …) now map to cross-supplier topics
- shop split ignores 1-2 stray rows instead of publishing a one-item list
- total 5,741 items across 29 price lists

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XoJGvA8cApVXFb92aBk3Fg
</commit_message>
<xml_diff>
--- a/downloads/shop.xlsx
+++ b/downloads/shop.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,7 +548,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Hill's Prescription Diet</t>
+          <t>פורינה (חנויות)</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -561,24 +561,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>פורינה (חנויות)</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>נוסחה: עלות = מחיר ללא מע"מ × (1 − הנחה) × 1.18 ; מחיר ללקוח = עלות × (1 + מרווח %) + מרווח ₪</t>
         </is>
@@ -595,7 +579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L381"/>
+  <dimension ref="A1:L379"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -19096,12 +19080,12 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>Hill's Prescription Diet</t>
+          <t>פורינה (חנויות)</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>חטיף היפואלרגני</t>
+          <t>פריסקיז פארטי מיקס אוריגי'נל קראנץ</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -19109,16 +19093,21 @@
           <t>חטיפים</t>
         </is>
       </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>12348261</t>
+        </is>
+      </c>
       <c r="E350" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F350" t="n">
-        <v>24</v>
+        <v>8.18</v>
       </c>
       <c r="G350" t="n">
-        <v>28.32</v>
+        <v>9.65</v>
       </c>
       <c r="H350">
         <f>הגדרות!B8</f>
@@ -19144,12 +19133,12 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>Hill's Prescription Diet</t>
+          <t>פורינה (חנויות)</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>חטיף שמירה על המשקל</t>
+          <t>פריסקיז פארטי מיקס מיקס גריל קראנץ</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -19157,16 +19146,21 @@
           <t>חטיפים</t>
         </is>
       </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>12348037</t>
+        </is>
+      </c>
       <c r="E351" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F351" t="n">
-        <v>21</v>
+        <v>8.18</v>
       </c>
       <c r="G351" t="n">
-        <v>24.78</v>
+        <v>9.65</v>
       </c>
       <c r="H351">
         <f>הגדרות!B8</f>
@@ -19197,7 +19191,7 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס אוריגי'נל קראנץ</t>
+          <t>פריסקיז פארטי מיקס מעדני ים קראנץ</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -19207,7 +19201,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>12348261</t>
+          <t>12364507</t>
         </is>
       </c>
       <c r="E352" t="inlineStr">
@@ -19222,7 +19216,7 @@
         <v>9.65</v>
       </c>
       <c r="H352">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I352">
@@ -19230,11 +19224,11 @@
         <v/>
       </c>
       <c r="J352">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K352">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L352">
@@ -19250,7 +19244,7 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס מיקס גריל קראנץ</t>
+          <t>פריסקיז פארטי מיקס פיקניק קרנץ</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -19260,7 +19254,7 @@
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>12348037</t>
+          <t>12368621</t>
         </is>
       </c>
       <c r="E353" t="inlineStr">
@@ -19275,7 +19269,7 @@
         <v>9.65</v>
       </c>
       <c r="H353">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I353">
@@ -19283,11 +19277,11 @@
         <v/>
       </c>
       <c r="J353">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K353">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L353">
@@ -19303,7 +19297,7 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס מעדני ים קראנץ</t>
+          <t>פריסקיז פארטי מיקס קרייזי צ'יז</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -19313,7 +19307,7 @@
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>12364507</t>
+          <t>12528489</t>
         </is>
       </c>
       <c r="E354" t="inlineStr">
@@ -19328,7 +19322,7 @@
         <v>9.65</v>
       </c>
       <c r="H354">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I354">
@@ -19336,11 +19330,11 @@
         <v/>
       </c>
       <c r="J354">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K354">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L354">
@@ -19356,7 +19350,7 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס פיקניק קרנץ</t>
+          <t>פריסקיז פארטי מיקס מאנץ' בוקר</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -19366,7 +19360,7 @@
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>12368621</t>
+          <t>12280472</t>
         </is>
       </c>
       <c r="E355" t="inlineStr">
@@ -19381,7 +19375,7 @@
         <v>9.65</v>
       </c>
       <c r="H355">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I355">
@@ -19389,11 +19383,11 @@
         <v/>
       </c>
       <c r="J355">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K355">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L355">
@@ -19409,7 +19403,7 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס קרייזי צ'יז</t>
+          <t>פריסקיז פארטי מיקס הודו</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -19419,7 +19413,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>12528489</t>
+          <t>12332654</t>
         </is>
       </c>
       <c r="E356" t="inlineStr">
@@ -19434,7 +19428,7 @@
         <v>9.65</v>
       </c>
       <c r="H356">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I356">
@@ -19442,11 +19436,11 @@
         <v/>
       </c>
       <c r="J356">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K356">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L356">
@@ -19462,7 +19456,7 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס מאנץ' בוקר</t>
+          <t>פריסקיז פארטי מיקס עוף</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -19472,7 +19466,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>12280472</t>
+          <t>12332617</t>
         </is>
       </c>
       <c r="E357" t="inlineStr">
@@ -19487,7 +19481,7 @@
         <v>9.65</v>
       </c>
       <c r="H357">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I357">
@@ -19495,11 +19489,11 @@
         <v/>
       </c>
       <c r="J357">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K357">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L357">
@@ -19515,7 +19509,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס הודו</t>
+          <t>פריסקיז פלייפולס סלמון ושרימפס</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -19525,7 +19519,7 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>12332654</t>
+          <t>12534203</t>
         </is>
       </c>
       <c r="E358" t="inlineStr">
@@ -19540,7 +19534,7 @@
         <v>9.65</v>
       </c>
       <c r="H358">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I358">
@@ -19548,11 +19542,11 @@
         <v/>
       </c>
       <c r="J358">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K358">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L358">
@@ -19568,7 +19562,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס עוף</t>
+          <t>פריסקיז פלייפולס עוף וכבד</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -19578,7 +19572,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>12332617</t>
+          <t>12534194</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
@@ -19593,7 +19587,7 @@
         <v>9.65</v>
       </c>
       <c r="H359">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I359">
@@ -19601,11 +19595,11 @@
         <v/>
       </c>
       <c r="J359">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K359">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L359">
@@ -19621,7 +19615,7 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>פריסקיז פלייפולס סלמון ושרימפס</t>
+          <t>פריסקיז צנצנת פארטי מיקס מעדני ים קראנץ</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -19631,7 +19625,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>12534203</t>
+          <t>12364794</t>
         </is>
       </c>
       <c r="E360" t="inlineStr">
@@ -19640,13 +19634,13 @@
         </is>
       </c>
       <c r="F360" t="n">
-        <v>8.18</v>
+        <v>50.67</v>
       </c>
       <c r="G360" t="n">
-        <v>9.65</v>
+        <v>59.79</v>
       </c>
       <c r="H360">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I360">
@@ -19654,11 +19648,11 @@
         <v/>
       </c>
       <c r="J360">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K360">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L360">
@@ -19674,7 +19668,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>פריסקיז פלייפולס עוף וכבד</t>
+          <t>פריסקיז צנצנת פארטי מיקס אוריגי'נל קראנץ</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -19684,7 +19678,7 @@
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>12534194</t>
+          <t>12349730</t>
         </is>
       </c>
       <c r="E361" t="inlineStr">
@@ -19693,13 +19687,13 @@
         </is>
       </c>
       <c r="F361" t="n">
-        <v>8.18</v>
+        <v>50.67</v>
       </c>
       <c r="G361" t="n">
-        <v>9.65</v>
+        <v>59.79</v>
       </c>
       <c r="H361">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I361">
@@ -19707,11 +19701,11 @@
         <v/>
       </c>
       <c r="J361">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K361">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L361">
@@ -19727,7 +19721,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>פריסקיז צנצנת פארטי מיקס מעדני ים קראנץ</t>
+          <t>דנטלייף לכלב מגזע קטן</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -19737,7 +19731,7 @@
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>12364794</t>
+          <t>12606950</t>
         </is>
       </c>
       <c r="E362" t="inlineStr">
@@ -19746,13 +19740,13 @@
         </is>
       </c>
       <c r="F362" t="n">
-        <v>50.67</v>
+        <v>10.2</v>
       </c>
       <c r="G362" t="n">
-        <v>59.79</v>
+        <v>12.04</v>
       </c>
       <c r="H362">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I362">
@@ -19760,11 +19754,11 @@
         <v/>
       </c>
       <c r="J362">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K362">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L362">
@@ -19780,7 +19774,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>פריסקיז צנצנת פארטי מיקס אוריגי'נל קראנץ</t>
+          <t>דנטלייף לכלב מגזע בינוני</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -19790,7 +19784,7 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>12349730</t>
+          <t>12606926</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
@@ -19799,13 +19793,13 @@
         </is>
       </c>
       <c r="F363" t="n">
-        <v>50.67</v>
+        <v>10.2</v>
       </c>
       <c r="G363" t="n">
-        <v>59.79</v>
+        <v>12.04</v>
       </c>
       <c r="H363">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I363">
@@ -19813,11 +19807,11 @@
         <v/>
       </c>
       <c r="J363">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K363">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L363">
@@ -19833,7 +19827,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>דנטלייף לכלב מגזע קטן</t>
+          <t>דנטלייף לכלב מגזע גדול</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -19843,7 +19837,7 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>12606950</t>
+          <t>12606948</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
@@ -19858,7 +19852,7 @@
         <v>12.04</v>
       </c>
       <c r="H364">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I364">
@@ -19866,11 +19860,11 @@
         <v/>
       </c>
       <c r="J364">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K364">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L364">
@@ -19886,7 +19880,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>דנטלייף לכלב מגזע בינוני</t>
+          <t>דנטלייף חתול עוף</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
@@ -19896,7 +19890,7 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>12606926</t>
+          <t>12607325</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
@@ -19905,13 +19899,13 @@
         </is>
       </c>
       <c r="F365" t="n">
-        <v>10.2</v>
+        <v>6.5</v>
       </c>
       <c r="G365" t="n">
-        <v>12.04</v>
+        <v>7.67</v>
       </c>
       <c r="H365">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I365">
@@ -19919,11 +19913,11 @@
         <v/>
       </c>
       <c r="J365">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K365">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L365">
@@ -19939,7 +19933,7 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>דנטלייף לכלב מגזע גדול</t>
+          <t>דנטלייף חתול סלמון</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -19949,7 +19943,7 @@
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>12606948</t>
+          <t>12607342</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
@@ -19958,13 +19952,13 @@
         </is>
       </c>
       <c r="F366" t="n">
-        <v>10.2</v>
+        <v>6.5</v>
       </c>
       <c r="G366" t="n">
-        <v>12.04</v>
+        <v>7.67</v>
       </c>
       <c r="H366">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I366">
@@ -19972,11 +19966,11 @@
         <v/>
       </c>
       <c r="J366">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K366">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L366">
@@ -19992,7 +19986,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>דנטלייף חתול עוף</t>
+          <t>פליקס שלוקים Joyables עוף</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -20002,7 +19996,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>12607325</t>
+          <t>12620437</t>
         </is>
       </c>
       <c r="E367" t="inlineStr">
@@ -20011,13 +20005,13 @@
         </is>
       </c>
       <c r="F367" t="n">
-        <v>6.5</v>
+        <v>8.49</v>
       </c>
       <c r="G367" t="n">
-        <v>7.67</v>
+        <v>10.02</v>
       </c>
       <c r="H367">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I367">
@@ -20025,11 +20019,11 @@
         <v/>
       </c>
       <c r="J367">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K367">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L367">
@@ -20045,7 +20039,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>דנטלייף חתול סלמון</t>
+          <t>פליקס שלוקים Joyables סלמון</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -20055,7 +20049,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>12607342</t>
+          <t>12620438</t>
         </is>
       </c>
       <c r="E368" t="inlineStr">
@@ -20064,13 +20058,13 @@
         </is>
       </c>
       <c r="F368" t="n">
-        <v>6.5</v>
+        <v>8.49</v>
       </c>
       <c r="G368" t="n">
-        <v>7.67</v>
+        <v>10.02</v>
       </c>
       <c r="H368">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I368">
@@ -20078,11 +20072,11 @@
         <v/>
       </c>
       <c r="J368">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K368">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L368">
@@ -20098,7 +20092,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>פליקס שלוקים Joyables עוף</t>
+          <t>פליקס שלוקים Joyables ברווז</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -20108,7 +20102,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>12620437</t>
+          <t>12620419</t>
         </is>
       </c>
       <c r="E369" t="inlineStr">
@@ -20123,7 +20117,7 @@
         <v>10.02</v>
       </c>
       <c r="H369">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I369">
@@ -20131,11 +20125,11 @@
         <v/>
       </c>
       <c r="J369">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K369">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L369">
@@ -20151,7 +20145,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>פליקס שלוקים Joyables סלמון</t>
+          <t>פרו פלאן חטיפי DentalCare לכלב מגזע קטן</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -20161,7 +20155,7 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>12620438</t>
+          <t>12604543</t>
         </is>
       </c>
       <c r="E370" t="inlineStr">
@@ -20170,13 +20164,13 @@
         </is>
       </c>
       <c r="F370" t="n">
-        <v>8.49</v>
+        <v>25.64</v>
       </c>
       <c r="G370" t="n">
-        <v>10.02</v>
+        <v>30.26</v>
       </c>
       <c r="H370">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I370">
@@ -20184,11 +20178,11 @@
         <v/>
       </c>
       <c r="J370">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K370">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L370">
@@ -20204,7 +20198,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>פליקס שלוקים Joyables ברווז</t>
+          <t>פרו פלאן חטיפי DentalCare לכלב מגזע בינוני</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -20214,7 +20208,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>12620419</t>
+          <t>12604772</t>
         </is>
       </c>
       <c r="E371" t="inlineStr">
@@ -20223,13 +20217,13 @@
         </is>
       </c>
       <c r="F371" t="n">
-        <v>8.49</v>
+        <v>25.64</v>
       </c>
       <c r="G371" t="n">
-        <v>10.02</v>
+        <v>30.26</v>
       </c>
       <c r="H371">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I371">
@@ -20237,11 +20231,11 @@
         <v/>
       </c>
       <c r="J371">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K371">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L371">
@@ -20257,7 +20251,7 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>פרו פלאן חטיפי DentalCare לכלב מגזע קטן</t>
+          <t>פרו פלאן חטיפי DentalCare לכלב מגזע גדול</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
@@ -20267,7 +20261,7 @@
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t>12604543</t>
+          <t>12604733</t>
         </is>
       </c>
       <c r="E372" t="inlineStr">
@@ -20282,7 +20276,7 @@
         <v>30.26</v>
       </c>
       <c r="H372">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I372">
@@ -20290,11 +20284,11 @@
         <v/>
       </c>
       <c r="J372">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K372">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L372">
@@ -20310,7 +20304,7 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>פרו פלאן חטיפי DentalCare לכלב מגזע בינוני</t>
+          <t>דוגלי אקטיב בקר</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -20320,7 +20314,7 @@
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>12604772</t>
+          <t>12466720</t>
         </is>
       </c>
       <c r="E373" t="inlineStr">
@@ -20329,13 +20323,13 @@
         </is>
       </c>
       <c r="F373" t="n">
-        <v>25.64</v>
+        <v>114.19</v>
       </c>
       <c r="G373" t="n">
-        <v>30.26</v>
+        <v>134.74</v>
       </c>
       <c r="H373">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I373">
@@ -20343,11 +20337,11 @@
         <v/>
       </c>
       <c r="J373">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K373">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L373">
@@ -20363,7 +20357,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>פרו פלאן חטיפי DentalCare לכלב מגזע גדול</t>
+          <t>דוגלי גורים עוף</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
@@ -20373,7 +20367,7 @@
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>12604733</t>
+          <t>12466622</t>
         </is>
       </c>
       <c r="E374" t="inlineStr">
@@ -20382,13 +20376,13 @@
         </is>
       </c>
       <c r="F374" t="n">
-        <v>25.64</v>
+        <v>41.46</v>
       </c>
       <c r="G374" t="n">
-        <v>30.26</v>
+        <v>48.92</v>
       </c>
       <c r="H374">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I374">
@@ -20396,11 +20390,11 @@
         <v/>
       </c>
       <c r="J374">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K374">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L374">
@@ -20416,7 +20410,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>דוגלי אקטיב בקר</t>
+          <t>דוגלי גזע קטן בקר</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -20426,7 +20420,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>12466720</t>
+          <t>12613172</t>
         </is>
       </c>
       <c r="E375" t="inlineStr">
@@ -20435,13 +20429,13 @@
         </is>
       </c>
       <c r="F375" t="n">
-        <v>114.19</v>
+        <v>39.49</v>
       </c>
       <c r="G375" t="n">
-        <v>134.74</v>
+        <v>46.6</v>
       </c>
       <c r="H375">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I375">
@@ -20449,11 +20443,11 @@
         <v/>
       </c>
       <c r="J375">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K375">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L375">
@@ -20469,7 +20463,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>דוגלי גורים עוף</t>
+          <t>דוגלי בוגר עוף</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -20479,7 +20473,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>12466622</t>
+          <t>12368765</t>
         </is>
       </c>
       <c r="E376" t="inlineStr">
@@ -20488,13 +20482,13 @@
         </is>
       </c>
       <c r="F376" t="n">
-        <v>41.46</v>
+        <v>37.61</v>
       </c>
       <c r="G376" t="n">
-        <v>48.92</v>
+        <v>44.38</v>
       </c>
       <c r="H376">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I376">
@@ -20502,11 +20496,11 @@
         <v/>
       </c>
       <c r="J376">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K376">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L376">
@@ -20522,7 +20516,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>דוגלי גזע קטן בקר</t>
+          <t>דוגלי בוגר בקר</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
@@ -20532,7 +20526,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>12613172</t>
+          <t>12368766</t>
         </is>
       </c>
       <c r="E377" t="inlineStr">
@@ -20541,13 +20535,13 @@
         </is>
       </c>
       <c r="F377" t="n">
-        <v>39.49</v>
+        <v>37.61</v>
       </c>
       <c r="G377" t="n">
-        <v>46.6</v>
+        <v>44.38</v>
       </c>
       <c r="H377">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I377">
@@ -20555,11 +20549,11 @@
         <v/>
       </c>
       <c r="J377">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K377">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L377">
@@ -20585,7 +20579,7 @@
       </c>
       <c r="D378" t="inlineStr">
         <is>
-          <t>12368765</t>
+          <t>12368676</t>
         </is>
       </c>
       <c r="E378" t="inlineStr">
@@ -20594,13 +20588,13 @@
         </is>
       </c>
       <c r="F378" t="n">
-        <v>37.61</v>
+        <v>108.76</v>
       </c>
       <c r="G378" t="n">
-        <v>44.38</v>
+        <v>128.34</v>
       </c>
       <c r="H378">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I378">
@@ -20608,11 +20602,11 @@
         <v/>
       </c>
       <c r="J378">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K378">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L378">
@@ -20638,7 +20632,7 @@
       </c>
       <c r="D379" t="inlineStr">
         <is>
-          <t>12368766</t>
+          <t>12368675</t>
         </is>
       </c>
       <c r="E379" t="inlineStr">
@@ -20647,13 +20641,13 @@
         </is>
       </c>
       <c r="F379" t="n">
-        <v>37.61</v>
+        <v>108.76</v>
       </c>
       <c r="G379" t="n">
-        <v>44.38</v>
+        <v>128.34</v>
       </c>
       <c r="H379">
-        <f>הגדרות!B9</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I379">
@@ -20661,121 +20655,15 @@
         <v/>
       </c>
       <c r="J379">
-        <f>הגדרות!C9</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K379">
-        <f>הגדרות!D9</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L379">
         <f>I379*(1+J379/100)+K379</f>
-        <v/>
-      </c>
-    </row>
-    <row r="380">
-      <c r="A380" t="inlineStr">
-        <is>
-          <t>פורינה (חנויות)</t>
-        </is>
-      </c>
-      <c r="B380" t="inlineStr">
-        <is>
-          <t>דוגלי בוגר עוף</t>
-        </is>
-      </c>
-      <c r="C380" t="inlineStr">
-        <is>
-          <t>חטיפים</t>
-        </is>
-      </c>
-      <c r="D380" t="inlineStr">
-        <is>
-          <t>12368676</t>
-        </is>
-      </c>
-      <c r="E380" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="F380" t="n">
-        <v>108.76</v>
-      </c>
-      <c r="G380" t="n">
-        <v>128.34</v>
-      </c>
-      <c r="H380">
-        <f>הגדרות!B9</f>
-        <v/>
-      </c>
-      <c r="I380">
-        <f>F380*(1-H380/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J380">
-        <f>הגדרות!C9</f>
-        <v/>
-      </c>
-      <c r="K380">
-        <f>הגדרות!D9</f>
-        <v/>
-      </c>
-      <c r="L380">
-        <f>I380*(1+J380/100)+K380</f>
-        <v/>
-      </c>
-    </row>
-    <row r="381">
-      <c r="A381" t="inlineStr">
-        <is>
-          <t>פורינה (חנויות)</t>
-        </is>
-      </c>
-      <c r="B381" t="inlineStr">
-        <is>
-          <t>דוגלי בוגר בקר</t>
-        </is>
-      </c>
-      <c r="C381" t="inlineStr">
-        <is>
-          <t>חטיפים</t>
-        </is>
-      </c>
-      <c r="D381" t="inlineStr">
-        <is>
-          <t>12368675</t>
-        </is>
-      </c>
-      <c r="E381" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="F381" t="n">
-        <v>108.76</v>
-      </c>
-      <c r="G381" t="n">
-        <v>128.34</v>
-      </c>
-      <c r="H381">
-        <f>הגדרות!B9</f>
-        <v/>
-      </c>
-      <c r="I381">
-        <f>F381*(1-H381/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J381">
-        <f>הגדרות!C9</f>
-        <v/>
-      </c>
-      <c r="K381">
-        <f>הגדרות!D9</f>
-        <v/>
-      </c>
-      <c r="L381">
-        <f>I381*(1+J381/100)+K381</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
data(vetmarket): build from parsed order confirmations only — there is no published price list
The clinic's vetmarket catalog (vetmarketCatalog.ts / "מחירון וטמרקט מלא.xlsx", 194 rows,
list price == net price on every row) is an internally maintained file, not a Vetmarket
publication, so it cannot back a price on a public site. It now supplies a category label
and nothing else; the 97 rows it was pricing are gone.

Every row is now the pre-discount unit price from an order confirmation, carrying its own
date (09/2023-08/2026), and a test asserts that invariant. The xlsx is no longer published
as a source file. 264 -> 171 rows; total 5,720.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XoJGvA8cApVXFb92aBk3Fg
</commit_message>
<xml_diff>
--- a/downloads/shop.xlsx
+++ b/downloads/shop.xlsx
@@ -579,7 +579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L379"/>
+  <dimension ref="A1:L376"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -15746,7 +15746,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>חטיף הילס היפואלרגני לכלב 200 גרם</t>
+          <t>תוסף מפרקים  DASUQUIN Nutramax חטיפים לכלב בינוני/קטן, 84 יח'</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -15756,7 +15756,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>40608557</t>
+          <t>181525</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -15765,10 +15765,10 @@
         </is>
       </c>
       <c r="F287" t="n">
-        <v>23</v>
+        <v>156</v>
       </c>
       <c r="G287" t="n">
-        <v>27.14</v>
+        <v>184.08</v>
       </c>
       <c r="H287">
         <f>הגדרות!B5</f>
@@ -15799,7 +15799,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>חטיף פודיס נגיסי סלמון 100 גרם</t>
+          <t>תוסף מפרקים  DASUQUIN Nutramax חטיפים לכלב גדול, 84 יח'</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -15809,7 +15809,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>48000004</t>
+          <t>181526</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -15818,10 +15818,10 @@
         </is>
       </c>
       <c r="F288" t="n">
-        <v>6</v>
+        <v>190</v>
       </c>
       <c r="G288" t="n">
-        <v>7.08</v>
+        <v>224.2</v>
       </c>
       <c r="H288">
         <f>הגדרות!B5</f>
@@ -15852,7 +15852,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>חטיף פודיס רצועות עוף רכות 100 גרם</t>
+          <t>חטיף FOODIES רצועות עוף רכות, 100 גרם</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -15905,7 +15905,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>חטיף פודיס נתחי ברווז רכים 100 גרם</t>
+          <t>חטיף FOODIES נגיסי סלמון, 100 גרם</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -15915,7 +15915,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>48000001</t>
+          <t>48000004</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -15924,10 +15924,10 @@
         </is>
       </c>
       <c r="F290" t="n">
-        <v>4.3</v>
+        <v>6</v>
       </c>
       <c r="G290" t="n">
-        <v>5.07</v>
+        <v>7.08</v>
       </c>
       <c r="H290">
         <f>הגדרות!B5</f>
@@ -15958,7 +15958,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>חטיף פודיס נגיסי ברווז 100 גרם</t>
+          <t>חטיף FOODIES נגיסי ברווז, 100 גרם</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -16011,17 +16011,17 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Kit4Cat חול</t>
+          <t>חטיף FOODIES גלילת ברווז עם עצם דנטלית 100 גרם</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>חול ושירותים</t>
+          <t>חטיפים</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>460001</t>
+          <t>48000013</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -16030,10 +16030,10 @@
         </is>
       </c>
       <c r="F292" t="n">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="G292" t="n">
-        <v>41.3</v>
+        <v>7.08</v>
       </c>
       <c r="H292">
         <f>הגדרות!B5</f>
@@ -16064,7 +16064,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>תוסף מפרקים  DASUQUIN Nutramax חטיפים לכלב בינוני/קטן, 84 יח'</t>
+          <t>חטיף FOODIES גלילת כבש, אורז ועור בקר, 100 גרם</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -16074,7 +16074,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>181525</t>
+          <t>48000015</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -16083,10 +16083,10 @@
         </is>
       </c>
       <c r="F293" t="n">
-        <v>156</v>
+        <v>6</v>
       </c>
       <c r="G293" t="n">
-        <v>184.08</v>
+        <v>7.08</v>
       </c>
       <c r="H293">
         <f>הגדרות!B5</f>
@@ -16117,7 +16117,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>תוסף מפרקים  DASUQUIN Nutramax חטיפים לכלב גדול, 84 יח'</t>
+          <t>חטיף FOODIES מקלות לעיסה עוף ועור בקר 1 ק"ג</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -16127,7 +16127,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>181526</t>
+          <t>48000025</t>
         </is>
       </c>
       <c r="E294" t="inlineStr">
@@ -16136,10 +16136,10 @@
         </is>
       </c>
       <c r="F294" t="n">
-        <v>190</v>
+        <v>53</v>
       </c>
       <c r="G294" t="n">
-        <v>224.2</v>
+        <v>62.54</v>
       </c>
       <c r="H294">
         <f>הגדרות!B5</f>
@@ -16170,7 +16170,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>חטיף FOODIES גלילת ברווז עם עצם דנטלית 100 גרם</t>
+          <t>חטיף FOODIES גלילת עוף ועור בקר ג'מבו 1 ק"ג</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -16180,7 +16180,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>48000013</t>
+          <t>48000027</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -16189,10 +16189,10 @@
         </is>
       </c>
       <c r="F295" t="n">
-        <v>6</v>
+        <v>53</v>
       </c>
       <c r="G295" t="n">
-        <v>7.08</v>
+        <v>62.54</v>
       </c>
       <c r="H295">
         <f>הגדרות!B5</f>
@@ -16223,7 +16223,7 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>חטיף FOODIES גלילת כבש, אורז ועור בקר, 100 גרם</t>
+          <t>חטיף FOODIES גלילת ברווז עם עצם סידן 1 ק"ג</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -16233,7 +16233,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>48000015</t>
+          <t>48000028</t>
         </is>
       </c>
       <c r="E296" t="inlineStr">
@@ -16242,10 +16242,10 @@
         </is>
       </c>
       <c r="F296" t="n">
-        <v>6</v>
+        <v>53</v>
       </c>
       <c r="G296" t="n">
-        <v>7.08</v>
+        <v>62.54</v>
       </c>
       <c r="H296">
         <f>הגדרות!B5</f>
@@ -16276,7 +16276,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>חטיף FOODIES מקלות לעיסה עוף ועור בקר 1 ק"ג</t>
+          <t>חטיף FOODIES פילה חזה עוף 1 ק"ג</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -16286,7 +16286,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>48000025</t>
+          <t>48000029</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -16329,7 +16329,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>חטיף FOODIES גלילת עוף ועור בקר ג'מבו 1 ק"ג</t>
+          <t>ק"ג 1 חטיף פודיס ברווז על מקלוני עור בקר,</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -16339,7 +16339,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>48000027</t>
+          <t>48000030</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -16382,7 +16382,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>חטיף FOODIES גלילת ברווז עם עצם סידן 1 ק"ג</t>
+          <t>חטיף FOODIES גלילת כבש ועור בקר, 1 ק"ג</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -16392,7 +16392,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>48000028</t>
+          <t>48000031</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -16435,7 +16435,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>חטיף FOODIES פילה חזה עוף 1 ק"ג</t>
+          <t>ק"ג 1 חטיף פודיס מקלות לעיסה כבש ועור בקר,</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -16445,7 +16445,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>48000029</t>
+          <t>48000032</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -16488,7 +16488,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>ק"ג 1 חטיף פודיס ברווז על מקלוני עור בקר,</t>
+          <t>חטיף FOODIES מקלות לעיסה סלמון ועור בקר, 1 ק"ג</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -16498,7 +16498,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>48000030</t>
+          <t>48000033</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -16536,37 +16536,37 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>וטמרקט</t>
+          <t>מדי-מרקט</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>חטיף FOODIES גלילת כבש ועור בקר, 1 ק"ג</t>
+          <t>@ סדיניה 35 60X90 יח' TENA BED @</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>חטיפים</t>
+          <t>אביזרים</t>
         </is>
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>48000031</t>
+          <t>33262-1</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F302" t="n">
-        <v>53</v>
+        <v>31.36</v>
       </c>
       <c r="G302" t="n">
-        <v>62.54</v>
+        <v>37</v>
       </c>
       <c r="H302">
-        <f>הגדרות!B5</f>
+        <f>הגדרות!B6</f>
         <v/>
       </c>
       <c r="I302">
@@ -16574,11 +16574,11 @@
         <v/>
       </c>
       <c r="J302">
-        <f>הגדרות!C5</f>
+        <f>הגדרות!C6</f>
         <v/>
       </c>
       <c r="K302">
-        <f>הגדרות!D5</f>
+        <f>הגדרות!D6</f>
         <v/>
       </c>
       <c r="L302">
@@ -16589,37 +16589,37 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>וטמרקט</t>
+          <t>מדי-מרקט</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>ק"ג 1 חטיף פודיס מקלות לעיסה כבש ועור בקר,</t>
+          <t>ANTIGONE WIPES 19*20 500</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>חטיפים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>48000032</t>
+          <t>M0002020</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F303" t="n">
-        <v>53</v>
+        <v>71.42</v>
       </c>
       <c r="G303" t="n">
-        <v>62.54</v>
+        <v>84.27</v>
       </c>
       <c r="H303">
-        <f>הגדרות!B5</f>
+        <f>הגדרות!B6</f>
         <v/>
       </c>
       <c r="I303">
@@ -16627,11 +16627,11 @@
         <v/>
       </c>
       <c r="J303">
-        <f>הגדרות!C5</f>
+        <f>הגדרות!C6</f>
         <v/>
       </c>
       <c r="K303">
-        <f>הגדרות!D5</f>
+        <f>הגדרות!D6</f>
         <v/>
       </c>
       <c r="L303">
@@ -16642,37 +16642,37 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>וטמרקט</t>
+          <t>מדי-מרקט</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>חטיף FOODIES מקלות לעיסה סלמון ועור בקר, 1 ק"ג</t>
+          <t>ANTIGONE WIPES 20*20 200</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>חטיפים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>48000033</t>
+          <t>100003</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F304" t="n">
-        <v>53</v>
+        <v>30.32</v>
       </c>
       <c r="G304" t="n">
-        <v>62.54</v>
+        <v>35.78</v>
       </c>
       <c r="H304">
-        <f>הגדרות!B5</f>
+        <f>הגדרות!B6</f>
         <v/>
       </c>
       <c r="I304">
@@ -16680,11 +16680,11 @@
         <v/>
       </c>
       <c r="J304">
-        <f>הגדרות!C5</f>
+        <f>הגדרות!C6</f>
         <v/>
       </c>
       <c r="K304">
-        <f>הגדרות!D5</f>
+        <f>הגדרות!D6</f>
         <v/>
       </c>
       <c r="L304">
@@ -16700,17 +16700,17 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>@ סדיניה 35 60X90 יח' TENA BED @</t>
+          <t>CETRIN 1 LITTER SOL</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>אביזרים</t>
+          <t>חול ושירותים</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>33262-1</t>
+          <t>33365</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
@@ -16719,10 +16719,10 @@
         </is>
       </c>
       <c r="F305" t="n">
-        <v>31.36</v>
+        <v>30.84</v>
       </c>
       <c r="G305" t="n">
-        <v>37</v>
+        <v>36.39</v>
       </c>
       <c r="H305">
         <f>הגדרות!B6</f>
@@ -16753,7 +16753,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>ANTIGONE WIPES 19*20 500</t>
+          <t>DOUXO S3 CALM MOUSSE 150 ML</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -16763,7 +16763,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>M0002020</t>
+          <t>81-105</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
@@ -16772,10 +16772,10 @@
         </is>
       </c>
       <c r="F306" t="n">
-        <v>71.42</v>
+        <v>58.47</v>
       </c>
       <c r="G306" t="n">
-        <v>84.27</v>
+        <v>69</v>
       </c>
       <c r="H306">
         <f>הגדרות!B6</f>
@@ -16806,7 +16806,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>ANTIGONE WIPES 20*20 200</t>
+          <t>DOUXO S3 PYO MOUSSE 150 ML</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -16816,7 +16816,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>100003</t>
+          <t>81-101</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -16825,10 +16825,10 @@
         </is>
       </c>
       <c r="F307" t="n">
-        <v>30.32</v>
+        <v>58.47</v>
       </c>
       <c r="G307" t="n">
-        <v>35.78</v>
+        <v>69</v>
       </c>
       <c r="H307">
         <f>הגדרות!B6</f>
@@ -16859,17 +16859,17 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>CETRIN 1 LITTER SOL</t>
+          <t>DOUXO S3 PYO PADS</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>חול ושירותים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>33365</t>
+          <t>81-107</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -16878,10 +16878,10 @@
         </is>
       </c>
       <c r="F308" t="n">
-        <v>30.84</v>
+        <v>36.44</v>
       </c>
       <c r="G308" t="n">
-        <v>36.39</v>
+        <v>43</v>
       </c>
       <c r="H308">
         <f>הגדרות!B6</f>
@@ -16912,7 +16912,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>DOUXO S3 CALM MOUSSE 150 ML</t>
+          <t>DOUXO S3 SEB MOUSSE 150 ML</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -16922,7 +16922,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>81-105</t>
+          <t>81-103</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -16965,17 +16965,17 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>DOUXO S3 PYO MOUSSE 150 ML</t>
+          <t>Easy Go 500 Litter - איזי גו</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>חול ושירותים</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>81-101</t>
+          <t>18033-1</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -16984,10 +16984,10 @@
         </is>
       </c>
       <c r="F310" t="n">
-        <v>58.47</v>
+        <v>14.32</v>
       </c>
       <c r="G310" t="n">
-        <v>69</v>
+        <v>16.9</v>
       </c>
       <c r="H310">
         <f>הגדרות!B6</f>
@@ -17018,17 +17018,17 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>DOUXO S3 PYO PADS</t>
+          <t>Pinchers 45chews peanut butter pill hiding treat</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>חטיפים</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>81-107</t>
+          <t>090062J.045</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -17037,10 +17037,10 @@
         </is>
       </c>
       <c r="F311" t="n">
-        <v>36.44</v>
+        <v>22.3</v>
       </c>
       <c r="G311" t="n">
-        <v>43</v>
+        <v>26.31</v>
       </c>
       <c r="H311">
         <f>הגדרות!B6</f>
@@ -17071,17 +17071,17 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>DOUXO S3 SEB MOUSSE 150 ML</t>
+          <t>אלונקה רכה מתקפלת NAR QuikLitter</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>חול ושירותים</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>81-103</t>
+          <t>4105</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -17090,10 +17090,10 @@
         </is>
       </c>
       <c r="F312" t="n">
-        <v>58.47</v>
+        <v>194.49</v>
       </c>
       <c r="G312" t="n">
-        <v>69</v>
+        <v>229.5</v>
       </c>
       <c r="H312">
         <f>הגדרות!B6</f>
@@ -17124,17 +17124,17 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Easy Go 500 Litter - איזי גו</t>
+          <t>כלוב נשיאה אטלס 10 ללא מזרון Ferplast</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>חול ושירותים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>18033-1</t>
+          <t>5550279</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -17143,10 +17143,10 @@
         </is>
       </c>
       <c r="F313" t="n">
-        <v>14.32</v>
+        <v>50.85</v>
       </c>
       <c r="G313" t="n">
-        <v>16.9</v>
+        <v>60</v>
       </c>
       <c r="H313">
         <f>הגדרות!B6</f>
@@ -17177,17 +17177,17 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Pinchers 45chews peanut butter pill hiding treat</t>
+          <t>כלוב נשיאה אטלס 20 ללא מזרון Ferplast</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>חטיפים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>090062J.045</t>
+          <t>5550280</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -17196,10 +17196,10 @@
         </is>
       </c>
       <c r="F314" t="n">
-        <v>22.3</v>
+        <v>88.14</v>
       </c>
       <c r="G314" t="n">
-        <v>26.31</v>
+        <v>104</v>
       </c>
       <c r="H314">
         <f>הגדרות!B6</f>
@@ -17230,17 +17230,17 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>אלונקה רכה מתקפלת NAR QuikLitter</t>
+          <t>מברשת רחצת ידיים לפני ניתוח, סטר', מדיקפרו</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>חול ושירותים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>4105</t>
+          <t>3694</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -17249,10 +17249,10 @@
         </is>
       </c>
       <c r="F315" t="n">
-        <v>194.49</v>
+        <v>0.87</v>
       </c>
       <c r="G315" t="n">
-        <v>229.5</v>
+        <v>1.03</v>
       </c>
       <c r="H315">
         <f>הגדרות!B6</f>
@@ -17283,7 +17283,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>כלוב נשיאה אטלס 10 ללא מזרון Ferplast</t>
+          <t>מגבונים - Clinell sporicidal wipesn 1/6</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -17293,7 +17293,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>5550279</t>
+          <t>CS25</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -17302,10 +17302,10 @@
         </is>
       </c>
       <c r="F316" t="n">
-        <v>50.85</v>
+        <v>156.78</v>
       </c>
       <c r="G316" t="n">
-        <v>60</v>
+        <v>185</v>
       </c>
       <c r="H316">
         <f>הגדרות!B6</f>
@@ -17336,7 +17336,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>כלוב נשיאה אטלס 20 ללא מזרון Ferplast</t>
+          <t>מגבונים - Clinell Universal wipes clip pack 50</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -17346,7 +17346,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>5550280</t>
+          <t>11050</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -17355,10 +17355,10 @@
         </is>
       </c>
       <c r="F317" t="n">
-        <v>88.14</v>
+        <v>9.25</v>
       </c>
       <c r="G317" t="n">
-        <v>104</v>
+        <v>10.92</v>
       </c>
       <c r="H317">
         <f>הגדרות!B6</f>
@@ -17389,7 +17389,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>מברשת רחצת ידיים לפני ניתוח, סטר', מדיקפרו</t>
+          <t>מגבונים - Clinell Universal Wipes pack of 200</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -17399,7 +17399,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>3694</t>
+          <t>11200</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -17408,10 +17408,10 @@
         </is>
       </c>
       <c r="F318" t="n">
-        <v>0.87</v>
+        <v>19.92</v>
       </c>
       <c r="G318" t="n">
-        <v>1.03</v>
+        <v>23.5</v>
       </c>
       <c r="H318">
         <f>הגדרות!B6</f>
@@ -17442,7 +17442,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>מגבונים - Clinell sporicidal wipesn 1/6</t>
+          <t>מגבונים מדי-קלין אקסטרה עבים מועשר באלוורה 500 יח 20X16 ס"מ</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -17452,7 +17452,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>CS25</t>
+          <t>128697</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -17461,10 +17461,10 @@
         </is>
       </c>
       <c r="F319" t="n">
-        <v>156.78</v>
+        <v>22.88</v>
       </c>
       <c r="G319" t="n">
-        <v>185</v>
+        <v>27</v>
       </c>
       <c r="H319">
         <f>הגדרות!B6</f>
@@ -17495,7 +17495,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>מגבונים - Clinell Universal wipes clip pack 50</t>
+          <t>מגבונים מדי-קלין מועשרים באלוורה 500 יח' 28X20 ס"מ</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -17505,7 +17505,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>11050</t>
+          <t>128695</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -17514,10 +17514,10 @@
         </is>
       </c>
       <c r="F320" t="n">
-        <v>9.25</v>
+        <v>22.88</v>
       </c>
       <c r="G320" t="n">
-        <v>10.92</v>
+        <v>27</v>
       </c>
       <c r="H320">
         <f>הגדרות!B6</f>
@@ -17548,17 +17548,17 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>מגבונים - Clinell Universal Wipes pack of 200</t>
+          <t>מיטה חשמלית דגם GUESS 402 מעקה מגלוון</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>אביזרים</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>11200</t>
+          <t>883135</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -17567,10 +17567,10 @@
         </is>
       </c>
       <c r="F321" t="n">
-        <v>19.92</v>
+        <v>6288.14</v>
       </c>
       <c r="G321" t="n">
-        <v>23.5</v>
+        <v>7420</v>
       </c>
       <c r="H321">
         <f>הגדרות!B6</f>
@@ -17601,7 +17601,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>מגבונים מדי-קלין אקסטרה עבים מועשר באלוורה 500 יח 20X16 ס"מ</t>
+          <t>מספריים אל חלד לציפורניים REISZ</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -17611,7 +17611,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>128697</t>
+          <t>434457</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -17620,10 +17620,10 @@
         </is>
       </c>
       <c r="F322" t="n">
-        <v>22.88</v>
+        <v>21.17</v>
       </c>
       <c r="G322" t="n">
-        <v>27</v>
+        <v>24.98</v>
       </c>
       <c r="H322">
         <f>הגדרות!B6</f>
@@ -17654,7 +17654,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>מגבונים מדי-קלין מועשרים באלוורה 500 יח' 28X20 ס"מ</t>
+          <t>משושת ג'ל 500 מ"ל פוליגונום רב תכליתי Herbaderm</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -17664,7 +17664,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>128695</t>
+          <t>67-105</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -17673,10 +17673,10 @@
         </is>
       </c>
       <c r="F323" t="n">
-        <v>22.88</v>
+        <v>157.63</v>
       </c>
       <c r="G323" t="n">
-        <v>27</v>
+        <v>186</v>
       </c>
       <c r="H323">
         <f>הגדרות!B6</f>
@@ -17707,17 +17707,17 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>מיטה חשמלית דגם GUESS 402 מעקה מגלוון</t>
+          <t>משושת קרם 500 מ"ל פוליגונום רב תכליתי Herbaderm</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>אביזרים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>883135</t>
+          <t>67-103</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -17726,10 +17726,10 @@
         </is>
       </c>
       <c r="F324" t="n">
-        <v>6288.14</v>
+        <v>157.63</v>
       </c>
       <c r="G324" t="n">
-        <v>7420</v>
+        <v>186</v>
       </c>
       <c r="H324">
         <f>הגדרות!B6</f>
@@ -17760,7 +17760,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>מספריים אל חלד לציפורניים REISZ</t>
+          <t>נייר לניגוב עדשות מיקרוסקופ 1159 1/280 Kimwipes</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -17770,7 +17770,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>434457</t>
+          <t>3422</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -17779,10 +17779,10 @@
         </is>
       </c>
       <c r="F325" t="n">
-        <v>21.17</v>
+        <v>26.44</v>
       </c>
       <c r="G325" t="n">
-        <v>24.98</v>
+        <v>31.2</v>
       </c>
       <c r="H325">
         <f>הגדרות!B6</f>
@@ -17813,17 +17813,17 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>משושת ג'ל 500 מ"ל פוליגונום רב תכליתי Herbaderm</t>
+          <t>סיר לילה פלסטיק/ מיטה גדול עם ידית, מדיקפרו</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>אביזרים</t>
         </is>
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>67-105</t>
+          <t>4055</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -17832,10 +17832,10 @@
         </is>
       </c>
       <c r="F326" t="n">
-        <v>157.63</v>
+        <v>11.86</v>
       </c>
       <c r="G326" t="n">
-        <v>186</v>
+        <v>14</v>
       </c>
       <c r="H326">
         <f>הגדרות!B6</f>
@@ -17866,7 +17866,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>משושת קרם 500 מ"ל פוליגונום רב תכליתי Herbaderm</t>
+          <t>קוצץ ציפורניים, מדיקפרו</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -17876,7 +17876,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>67-103</t>
+          <t>17709</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -17885,10 +17885,10 @@
         </is>
       </c>
       <c r="F327" t="n">
-        <v>157.63</v>
+        <v>3.32</v>
       </c>
       <c r="G327" t="n">
-        <v>186</v>
+        <v>3.92</v>
       </c>
       <c r="H327">
         <f>הגדרות!B6</f>
@@ -17919,7 +17919,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>נייר לניגוב עדשות מיקרוסקופ 1159 1/280 Kimwipes</t>
+          <t>ראש למכונת תספורת (סכין) 40 - 0.25 מ"מ LAUBE</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -17929,7 +17929,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>3422</t>
+          <t>80662</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -17938,10 +17938,10 @@
         </is>
       </c>
       <c r="F328" t="n">
-        <v>26.44</v>
+        <v>120.13</v>
       </c>
       <c r="G328" t="n">
-        <v>31.2</v>
+        <v>141.75</v>
       </c>
       <c r="H328">
         <f>הגדרות!B6</f>
@@ -17972,7 +17972,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>סיר לילה פלסטיק/ מיטה גדול עם ידית, מדיקפרו</t>
+          <t>רצועה ללוח גב צבע כתום עם אבזם מתכת</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -17982,7 +17982,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>4055</t>
+          <t>16155</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -17991,10 +17991,10 @@
         </is>
       </c>
       <c r="F329" t="n">
-        <v>11.86</v>
+        <v>71.19</v>
       </c>
       <c r="G329" t="n">
-        <v>14</v>
+        <v>84</v>
       </c>
       <c r="H329">
         <f>הגדרות!B6</f>
@@ -18025,17 +18025,17 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>קוצץ ציפורניים, מדיקפרו</t>
+          <t>רצועה לתמיכה למסכת טרכוסטומי L</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>אביזרים</t>
         </is>
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>17709</t>
+          <t>7985</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -18044,10 +18044,10 @@
         </is>
       </c>
       <c r="F330" t="n">
-        <v>3.32</v>
+        <v>5.91</v>
       </c>
       <c r="G330" t="n">
-        <v>3.92</v>
+        <v>6.97</v>
       </c>
       <c r="H330">
         <f>הגדרות!B6</f>
@@ -18078,17 +18078,17 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>ראש למכונת תספורת (סכין) 40 - 0.25 מ"מ LAUBE</t>
+          <t>רצועה לתמיכה למסכת טרכוסטומי M</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>אביזרים</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>80662</t>
+          <t>7987</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -18097,10 +18097,10 @@
         </is>
       </c>
       <c r="F331" t="n">
-        <v>120.13</v>
+        <v>6.19</v>
       </c>
       <c r="G331" t="n">
-        <v>141.75</v>
+        <v>7.3</v>
       </c>
       <c r="H331">
         <f>הגדרות!B6</f>
@@ -18131,7 +18131,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>רצועה ללוח גב צבע כתום עם אבזם מתכת</t>
+          <t>רצועה לתמיכה למסכת טרכוסטומי XL</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -18141,7 +18141,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>16155</t>
+          <t>7986</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -18150,10 +18150,10 @@
         </is>
       </c>
       <c r="F332" t="n">
-        <v>71.19</v>
+        <v>6.36</v>
       </c>
       <c r="G332" t="n">
-        <v>84</v>
+        <v>7.5</v>
       </c>
       <c r="H332">
         <f>הגדרות!B6</f>
@@ -18179,37 +18179,37 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>מדי-מרקט</t>
+          <t>פט-וט ביומד</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>רצועה לתמיכה למסכת טרכוסטומי L</t>
+          <t>Keto Tris Finger Wipes 50 units</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>אביזרים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>7985</t>
+          <t>DERMA-SP1330</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="F333" t="n">
-        <v>5.91</v>
+        <v>59</v>
       </c>
       <c r="G333" t="n">
-        <v>6.97</v>
+        <v>69.62</v>
       </c>
       <c r="H333">
-        <f>הגדרות!B6</f>
+        <f>הגדרות!B7</f>
         <v/>
       </c>
       <c r="I333">
@@ -18217,11 +18217,11 @@
         <v/>
       </c>
       <c r="J333">
-        <f>הגדרות!C6</f>
+        <f>הגדרות!C7</f>
         <v/>
       </c>
       <c r="K333">
-        <f>הגדרות!D6</f>
+        <f>הגדרות!D7</f>
         <v/>
       </c>
       <c r="L333">
@@ -18232,37 +18232,37 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>מדי-מרקט</t>
+          <t>פט-וט ביומד</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>רצועה לתמיכה למסכת טרכוסטומי M</t>
+          <t>Tris Ophto Wipes 50ct</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>אביזרים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>7987</t>
+          <t>DZOO-TWX</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="F334" t="n">
-        <v>6.19</v>
+        <v>58</v>
       </c>
       <c r="G334" t="n">
-        <v>7.3</v>
+        <v>68.44</v>
       </c>
       <c r="H334">
-        <f>הגדרות!B6</f>
+        <f>הגדרות!B7</f>
         <v/>
       </c>
       <c r="I334">
@@ -18270,11 +18270,11 @@
         <v/>
       </c>
       <c r="J334">
-        <f>הגדרות!C6</f>
+        <f>הגדרות!C7</f>
         <v/>
       </c>
       <c r="K334">
-        <f>הגדרות!D6</f>
+        <f>הגדרות!D7</f>
         <v/>
       </c>
       <c r="L334">
@@ -18285,37 +18285,37 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>מדי-מרקט</t>
+          <t>פט-וט ביומד</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>רצועה לתמיכה למסכת טרכוסטומי XL</t>
+          <t>Pill Splitter</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>אביזרים</t>
+          <t>חול ושירותים</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>7986</t>
+          <t>FIONA-821070-1</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="F335" t="n">
-        <v>6.36</v>
+        <v>7</v>
       </c>
       <c r="G335" t="n">
-        <v>7.5</v>
+        <v>8.26</v>
       </c>
       <c r="H335">
-        <f>הגדרות!B6</f>
+        <f>הגדרות!B7</f>
         <v/>
       </c>
       <c r="I335">
@@ -18323,11 +18323,11 @@
         <v/>
       </c>
       <c r="J335">
-        <f>הגדרות!C6</f>
+        <f>הגדרות!C7</f>
         <v/>
       </c>
       <c r="K335">
-        <f>הגדרות!D6</f>
+        <f>הגדרות!D7</f>
         <v/>
       </c>
       <c r="L335">
@@ -18343,17 +18343,17 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Keto Tris Finger Wipes 50 units</t>
+          <t>Calming Spray 200ml</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>הרגעה</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>DERMA-SP1330</t>
+          <t>PR-79583</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -18362,10 +18362,10 @@
         </is>
       </c>
       <c r="F336" t="n">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="G336" t="n">
-        <v>69.62</v>
+        <v>54.28</v>
       </c>
       <c r="H336">
         <f>הגדרות!B7</f>
@@ -18396,17 +18396,17 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Tris Ophto Wipes 50ct</t>
+          <t>Mini Calming Spray 15ml</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>הרגעה</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>DZOO-TWX</t>
+          <t>PR-79664</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -18415,10 +18415,10 @@
         </is>
       </c>
       <c r="F337" t="n">
-        <v>58</v>
+        <v>18</v>
       </c>
       <c r="G337" t="n">
-        <v>68.44</v>
+        <v>21.24</v>
       </c>
       <c r="H337">
         <f>הגדרות!B7</f>
@@ -18449,17 +18449,17 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Pill Splitter</t>
+          <t>Battery Atomizer Refill 300ml</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>חול ושירותים</t>
+          <t>הרגעה</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>FIONA-821070-1</t>
+          <t>PR-79744</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -18468,10 +18468,10 @@
         </is>
       </c>
       <c r="F338" t="n">
-        <v>7</v>
+        <v>56</v>
       </c>
       <c r="G338" t="n">
-        <v>8.26</v>
+        <v>66.08</v>
       </c>
       <c r="H338">
         <f>הגדרות!B7</f>
@@ -18502,7 +18502,7 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Calming Spray 200ml</t>
+          <t>Battery Atomizer</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -18512,7 +18512,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>PR-79583</t>
+          <t>PR-79745</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -18521,10 +18521,10 @@
         </is>
       </c>
       <c r="F339" t="n">
-        <v>46</v>
+        <v>185</v>
       </c>
       <c r="G339" t="n">
-        <v>54.28</v>
+        <v>218.3</v>
       </c>
       <c r="H339">
         <f>הגדרות!B7</f>
@@ -18555,7 +18555,7 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Mini Calming Spray 15ml</t>
+          <t>Calming Wipe Sachet (12)</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -18565,7 +18565,7 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>PR-79664</t>
+          <t>PR-79881</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
@@ -18608,17 +18608,17 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Battery Atomizer Refill 300ml</t>
+          <t>Boredom Buster forager kit</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>הרגעה</t>
+          <t>צעצועים</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>PR-79744</t>
+          <t>PR-80128</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
@@ -18627,10 +18627,10 @@
         </is>
       </c>
       <c r="F341" t="n">
-        <v>56</v>
+        <v>105</v>
       </c>
       <c r="G341" t="n">
-        <v>66.08</v>
+        <v>123.9</v>
       </c>
       <c r="H341">
         <f>הגדרות!B7</f>
@@ -18661,7 +18661,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Battery Atomizer</t>
+          <t>Calming Bandana Kit EXTRA SMALL</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -18671,7 +18671,7 @@
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>PR-79745</t>
+          <t>PR-79959</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
@@ -18680,10 +18680,10 @@
         </is>
       </c>
       <c r="F342" t="n">
-        <v>185</v>
+        <v>44</v>
       </c>
       <c r="G342" t="n">
-        <v>218.3</v>
+        <v>51.92</v>
       </c>
       <c r="H342">
         <f>הגדרות!B7</f>
@@ -18714,7 +18714,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Calming Wipe Sachet (12)</t>
+          <t>Calming Bandana Kit SMALL</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -18724,7 +18724,7 @@
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>PR-79881</t>
+          <t>PR-79960</t>
         </is>
       </c>
       <c r="E343" t="inlineStr">
@@ -18733,10 +18733,10 @@
         </is>
       </c>
       <c r="F343" t="n">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="G343" t="n">
-        <v>21.24</v>
+        <v>51.92</v>
       </c>
       <c r="H343">
         <f>הגדרות!B7</f>
@@ -18767,17 +18767,17 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Boredom Buster forager kit</t>
+          <t>Calming Bandana Kit MEDIUM</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>צעצועים</t>
+          <t>הרגעה</t>
         </is>
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>PR-80128</t>
+          <t>PR-79961</t>
         </is>
       </c>
       <c r="E344" t="inlineStr">
@@ -18786,10 +18786,10 @@
         </is>
       </c>
       <c r="F344" t="n">
-        <v>105</v>
+        <v>44</v>
       </c>
       <c r="G344" t="n">
-        <v>123.9</v>
+        <v>51.92</v>
       </c>
       <c r="H344">
         <f>הגדרות!B7</f>
@@ -18820,7 +18820,7 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Calming Bandana Kit EXTRA SMALL</t>
+          <t>Calming Bandana Kit LARGE</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -18830,7 +18830,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>PR-79959</t>
+          <t>PR-79962</t>
         </is>
       </c>
       <c r="E345" t="inlineStr">
@@ -18873,7 +18873,7 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Calming Bandana Kit SMALL</t>
+          <t>Calming Spray 400ml – PROF. PACK</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -18883,7 +18883,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>PR-79960</t>
+          <t>PR-79983</t>
         </is>
       </c>
       <c r="E346" t="inlineStr">
@@ -18892,10 +18892,10 @@
         </is>
       </c>
       <c r="F346" t="n">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="G346" t="n">
-        <v>51.92</v>
+        <v>71.98</v>
       </c>
       <c r="H346">
         <f>הגדרות!B7</f>
@@ -18921,37 +18921,37 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>פט-וט ביומד</t>
+          <t>פורינה (חנויות)</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Calming Bandana Kit MEDIUM</t>
+          <t>פריסקיז פארטי מיקס אוריגי'נל קראנץ</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>הרגעה</t>
+          <t>חטיפים</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>PR-79961</t>
+          <t>12348261</t>
         </is>
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F347" t="n">
-        <v>44</v>
+        <v>8.18</v>
       </c>
       <c r="G347" t="n">
-        <v>51.92</v>
+        <v>9.65</v>
       </c>
       <c r="H347">
-        <f>הגדרות!B7</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I347">
@@ -18959,11 +18959,11 @@
         <v/>
       </c>
       <c r="J347">
-        <f>הגדרות!C7</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K347">
-        <f>הגדרות!D7</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L347">
@@ -18974,37 +18974,37 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>פט-וט ביומד</t>
+          <t>פורינה (חנויות)</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Calming Bandana Kit LARGE</t>
+          <t>פריסקיז פארטי מיקס מיקס גריל קראנץ</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>הרגעה</t>
+          <t>חטיפים</t>
         </is>
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>PR-79962</t>
+          <t>12348037</t>
         </is>
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F348" t="n">
-        <v>44</v>
+        <v>8.18</v>
       </c>
       <c r="G348" t="n">
-        <v>51.92</v>
+        <v>9.65</v>
       </c>
       <c r="H348">
-        <f>הגדרות!B7</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I348">
@@ -19012,11 +19012,11 @@
         <v/>
       </c>
       <c r="J348">
-        <f>הגדרות!C7</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K348">
-        <f>הגדרות!D7</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L348">
@@ -19027,37 +19027,37 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>פט-וט ביומד</t>
+          <t>פורינה (חנויות)</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Calming Spray 400ml – PROF. PACK</t>
+          <t>פריסקיז פארטי מיקס מעדני ים קראנץ</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>הרגעה</t>
+          <t>חטיפים</t>
         </is>
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>PR-79983</t>
+          <t>12364507</t>
         </is>
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F349" t="n">
-        <v>61</v>
+        <v>8.18</v>
       </c>
       <c r="G349" t="n">
-        <v>71.98</v>
+        <v>9.65</v>
       </c>
       <c r="H349">
-        <f>הגדרות!B7</f>
+        <f>הגדרות!B8</f>
         <v/>
       </c>
       <c r="I349">
@@ -19065,11 +19065,11 @@
         <v/>
       </c>
       <c r="J349">
-        <f>הגדרות!C7</f>
+        <f>הגדרות!C8</f>
         <v/>
       </c>
       <c r="K349">
-        <f>הגדרות!D7</f>
+        <f>הגדרות!D8</f>
         <v/>
       </c>
       <c r="L349">
@@ -19085,7 +19085,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס אוריגי'נל קראנץ</t>
+          <t>פריסקיז פארטי מיקס פיקניק קרנץ</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -19095,7 +19095,7 @@
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>12348261</t>
+          <t>12368621</t>
         </is>
       </c>
       <c r="E350" t="inlineStr">
@@ -19138,7 +19138,7 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס מיקס גריל קראנץ</t>
+          <t>פריסקיז פארטי מיקס קרייזי צ'יז</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -19148,7 +19148,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>12348037</t>
+          <t>12528489</t>
         </is>
       </c>
       <c r="E351" t="inlineStr">
@@ -19191,7 +19191,7 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס מעדני ים קראנץ</t>
+          <t>פריסקיז פארטי מיקס מאנץ' בוקר</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -19201,7 +19201,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>12364507</t>
+          <t>12280472</t>
         </is>
       </c>
       <c r="E352" t="inlineStr">
@@ -19244,7 +19244,7 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס פיקניק קרנץ</t>
+          <t>פריסקיז פארטי מיקס הודו</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -19254,7 +19254,7 @@
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>12368621</t>
+          <t>12332654</t>
         </is>
       </c>
       <c r="E353" t="inlineStr">
@@ -19297,7 +19297,7 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס קרייזי צ'יז</t>
+          <t>פריסקיז פארטי מיקס עוף</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -19307,7 +19307,7 @@
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>12528489</t>
+          <t>12332617</t>
         </is>
       </c>
       <c r="E354" t="inlineStr">
@@ -19350,7 +19350,7 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס מאנץ' בוקר</t>
+          <t>פריסקיז פלייפולס סלמון ושרימפס</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -19360,7 +19360,7 @@
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>12280472</t>
+          <t>12534203</t>
         </is>
       </c>
       <c r="E355" t="inlineStr">
@@ -19403,7 +19403,7 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס הודו</t>
+          <t>פריסקיז פלייפולס עוף וכבד</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -19413,7 +19413,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>12332654</t>
+          <t>12534194</t>
         </is>
       </c>
       <c r="E356" t="inlineStr">
@@ -19456,7 +19456,7 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס עוף</t>
+          <t>פריסקיז צנצנת פארטי מיקס מעדני ים קראנץ</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -19466,7 +19466,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>12332617</t>
+          <t>12364794</t>
         </is>
       </c>
       <c r="E357" t="inlineStr">
@@ -19475,10 +19475,10 @@
         </is>
       </c>
       <c r="F357" t="n">
-        <v>8.18</v>
+        <v>50.67</v>
       </c>
       <c r="G357" t="n">
-        <v>9.65</v>
+        <v>59.79</v>
       </c>
       <c r="H357">
         <f>הגדרות!B8</f>
@@ -19509,7 +19509,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>פריסקיז פלייפולס סלמון ושרימפס</t>
+          <t>פריסקיז צנצנת פארטי מיקס אוריגי'נל קראנץ</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -19519,7 +19519,7 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>12534203</t>
+          <t>12349730</t>
         </is>
       </c>
       <c r="E358" t="inlineStr">
@@ -19528,10 +19528,10 @@
         </is>
       </c>
       <c r="F358" t="n">
-        <v>8.18</v>
+        <v>50.67</v>
       </c>
       <c r="G358" t="n">
-        <v>9.65</v>
+        <v>59.79</v>
       </c>
       <c r="H358">
         <f>הגדרות!B8</f>
@@ -19562,7 +19562,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>פריסקיז פלייפולס עוף וכבד</t>
+          <t>דנטלייף לכלב מגזע קטן</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -19572,7 +19572,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>12534194</t>
+          <t>12606950</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
@@ -19581,10 +19581,10 @@
         </is>
       </c>
       <c r="F359" t="n">
-        <v>8.18</v>
+        <v>10.2</v>
       </c>
       <c r="G359" t="n">
-        <v>9.65</v>
+        <v>12.04</v>
       </c>
       <c r="H359">
         <f>הגדרות!B8</f>
@@ -19615,7 +19615,7 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>פריסקיז צנצנת פארטי מיקס מעדני ים קראנץ</t>
+          <t>דנטלייף לכלב מגזע בינוני</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -19625,7 +19625,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>12364794</t>
+          <t>12606926</t>
         </is>
       </c>
       <c r="E360" t="inlineStr">
@@ -19634,10 +19634,10 @@
         </is>
       </c>
       <c r="F360" t="n">
-        <v>50.67</v>
+        <v>10.2</v>
       </c>
       <c r="G360" t="n">
-        <v>59.79</v>
+        <v>12.04</v>
       </c>
       <c r="H360">
         <f>הגדרות!B8</f>
@@ -19668,7 +19668,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>פריסקיז צנצנת פארטי מיקס אוריגי'נל קראנץ</t>
+          <t>דנטלייף לכלב מגזע גדול</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -19678,7 +19678,7 @@
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>12349730</t>
+          <t>12606948</t>
         </is>
       </c>
       <c r="E361" t="inlineStr">
@@ -19687,10 +19687,10 @@
         </is>
       </c>
       <c r="F361" t="n">
-        <v>50.67</v>
+        <v>10.2</v>
       </c>
       <c r="G361" t="n">
-        <v>59.79</v>
+        <v>12.04</v>
       </c>
       <c r="H361">
         <f>הגדרות!B8</f>
@@ -19721,7 +19721,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>דנטלייף לכלב מגזע קטן</t>
+          <t>דנטלייף חתול עוף</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -19731,7 +19731,7 @@
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>12606950</t>
+          <t>12607325</t>
         </is>
       </c>
       <c r="E362" t="inlineStr">
@@ -19740,10 +19740,10 @@
         </is>
       </c>
       <c r="F362" t="n">
-        <v>10.2</v>
+        <v>6.5</v>
       </c>
       <c r="G362" t="n">
-        <v>12.04</v>
+        <v>7.67</v>
       </c>
       <c r="H362">
         <f>הגדרות!B8</f>
@@ -19774,7 +19774,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>דנטלייף לכלב מגזע בינוני</t>
+          <t>דנטלייף חתול סלמון</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -19784,7 +19784,7 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>12606926</t>
+          <t>12607342</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
@@ -19793,10 +19793,10 @@
         </is>
       </c>
       <c r="F363" t="n">
-        <v>10.2</v>
+        <v>6.5</v>
       </c>
       <c r="G363" t="n">
-        <v>12.04</v>
+        <v>7.67</v>
       </c>
       <c r="H363">
         <f>הגדרות!B8</f>
@@ -19827,7 +19827,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>דנטלייף לכלב מגזע גדול</t>
+          <t>פליקס שלוקים Joyables עוף</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -19837,7 +19837,7 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>12606948</t>
+          <t>12620437</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
@@ -19846,10 +19846,10 @@
         </is>
       </c>
       <c r="F364" t="n">
-        <v>10.2</v>
+        <v>8.49</v>
       </c>
       <c r="G364" t="n">
-        <v>12.04</v>
+        <v>10.02</v>
       </c>
       <c r="H364">
         <f>הגדרות!B8</f>
@@ -19880,7 +19880,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>דנטלייף חתול עוף</t>
+          <t>פליקס שלוקים Joyables סלמון</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
@@ -19890,7 +19890,7 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>12607325</t>
+          <t>12620438</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
@@ -19899,10 +19899,10 @@
         </is>
       </c>
       <c r="F365" t="n">
-        <v>6.5</v>
+        <v>8.49</v>
       </c>
       <c r="G365" t="n">
-        <v>7.67</v>
+        <v>10.02</v>
       </c>
       <c r="H365">
         <f>הגדרות!B8</f>
@@ -19933,7 +19933,7 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>דנטלייף חתול סלמון</t>
+          <t>פליקס שלוקים Joyables ברווז</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -19943,7 +19943,7 @@
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>12607342</t>
+          <t>12620419</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
@@ -19952,10 +19952,10 @@
         </is>
       </c>
       <c r="F366" t="n">
-        <v>6.5</v>
+        <v>8.49</v>
       </c>
       <c r="G366" t="n">
-        <v>7.67</v>
+        <v>10.02</v>
       </c>
       <c r="H366">
         <f>הגדרות!B8</f>
@@ -19986,7 +19986,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>פליקס שלוקים Joyables עוף</t>
+          <t>פרו פלאן חטיפי DentalCare לכלב מגזע קטן</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -19996,7 +19996,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>12620437</t>
+          <t>12604543</t>
         </is>
       </c>
       <c r="E367" t="inlineStr">
@@ -20005,10 +20005,10 @@
         </is>
       </c>
       <c r="F367" t="n">
-        <v>8.49</v>
+        <v>25.64</v>
       </c>
       <c r="G367" t="n">
-        <v>10.02</v>
+        <v>30.26</v>
       </c>
       <c r="H367">
         <f>הגדרות!B8</f>
@@ -20039,7 +20039,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>פליקס שלוקים Joyables סלמון</t>
+          <t>פרו פלאן חטיפי DentalCare לכלב מגזע בינוני</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -20049,7 +20049,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>12620438</t>
+          <t>12604772</t>
         </is>
       </c>
       <c r="E368" t="inlineStr">
@@ -20058,10 +20058,10 @@
         </is>
       </c>
       <c r="F368" t="n">
-        <v>8.49</v>
+        <v>25.64</v>
       </c>
       <c r="G368" t="n">
-        <v>10.02</v>
+        <v>30.26</v>
       </c>
       <c r="H368">
         <f>הגדרות!B8</f>
@@ -20092,7 +20092,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>פליקס שלוקים Joyables ברווז</t>
+          <t>פרו פלאן חטיפי DentalCare לכלב מגזע גדול</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -20102,7 +20102,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>12620419</t>
+          <t>12604733</t>
         </is>
       </c>
       <c r="E369" t="inlineStr">
@@ -20111,10 +20111,10 @@
         </is>
       </c>
       <c r="F369" t="n">
-        <v>8.49</v>
+        <v>25.64</v>
       </c>
       <c r="G369" t="n">
-        <v>10.02</v>
+        <v>30.26</v>
       </c>
       <c r="H369">
         <f>הגדרות!B8</f>
@@ -20145,7 +20145,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>פרו פלאן חטיפי DentalCare לכלב מגזע קטן</t>
+          <t>דוגלי אקטיב בקר</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -20155,7 +20155,7 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>12604543</t>
+          <t>12466720</t>
         </is>
       </c>
       <c r="E370" t="inlineStr">
@@ -20164,10 +20164,10 @@
         </is>
       </c>
       <c r="F370" t="n">
-        <v>25.64</v>
+        <v>114.19</v>
       </c>
       <c r="G370" t="n">
-        <v>30.26</v>
+        <v>134.74</v>
       </c>
       <c r="H370">
         <f>הגדרות!B8</f>
@@ -20198,7 +20198,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>פרו פלאן חטיפי DentalCare לכלב מגזע בינוני</t>
+          <t>דוגלי גורים עוף</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -20208,7 +20208,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>12604772</t>
+          <t>12466622</t>
         </is>
       </c>
       <c r="E371" t="inlineStr">
@@ -20217,10 +20217,10 @@
         </is>
       </c>
       <c r="F371" t="n">
-        <v>25.64</v>
+        <v>41.46</v>
       </c>
       <c r="G371" t="n">
-        <v>30.26</v>
+        <v>48.92</v>
       </c>
       <c r="H371">
         <f>הגדרות!B8</f>
@@ -20251,7 +20251,7 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>פרו פלאן חטיפי DentalCare לכלב מגזע גדול</t>
+          <t>דוגלי גזע קטן בקר</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
@@ -20261,7 +20261,7 @@
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t>12604733</t>
+          <t>12613172</t>
         </is>
       </c>
       <c r="E372" t="inlineStr">
@@ -20270,10 +20270,10 @@
         </is>
       </c>
       <c r="F372" t="n">
-        <v>25.64</v>
+        <v>39.49</v>
       </c>
       <c r="G372" t="n">
-        <v>30.26</v>
+        <v>46.6</v>
       </c>
       <c r="H372">
         <f>הגדרות!B8</f>
@@ -20304,7 +20304,7 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>דוגלי אקטיב בקר</t>
+          <t>דוגלי בוגר עוף</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -20314,7 +20314,7 @@
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>12466720</t>
+          <t>12368765</t>
         </is>
       </c>
       <c r="E373" t="inlineStr">
@@ -20323,10 +20323,10 @@
         </is>
       </c>
       <c r="F373" t="n">
-        <v>114.19</v>
+        <v>37.61</v>
       </c>
       <c r="G373" t="n">
-        <v>134.74</v>
+        <v>44.38</v>
       </c>
       <c r="H373">
         <f>הגדרות!B8</f>
@@ -20357,7 +20357,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>דוגלי גורים עוף</t>
+          <t>דוגלי בוגר בקר</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
@@ -20367,7 +20367,7 @@
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>12466622</t>
+          <t>12368766</t>
         </is>
       </c>
       <c r="E374" t="inlineStr">
@@ -20376,10 +20376,10 @@
         </is>
       </c>
       <c r="F374" t="n">
-        <v>41.46</v>
+        <v>37.61</v>
       </c>
       <c r="G374" t="n">
-        <v>48.92</v>
+        <v>44.38</v>
       </c>
       <c r="H374">
         <f>הגדרות!B8</f>
@@ -20410,7 +20410,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>דוגלי גזע קטן בקר</t>
+          <t>דוגלי בוגר עוף</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -20420,7 +20420,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>12613172</t>
+          <t>12368676</t>
         </is>
       </c>
       <c r="E375" t="inlineStr">
@@ -20429,10 +20429,10 @@
         </is>
       </c>
       <c r="F375" t="n">
-        <v>39.49</v>
+        <v>108.76</v>
       </c>
       <c r="G375" t="n">
-        <v>46.6</v>
+        <v>128.34</v>
       </c>
       <c r="H375">
         <f>הגדרות!B8</f>
@@ -20463,7 +20463,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>דוגלי בוגר עוף</t>
+          <t>דוגלי בוגר בקר</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -20473,7 +20473,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>12368765</t>
+          <t>12368675</t>
         </is>
       </c>
       <c r="E376" t="inlineStr">
@@ -20482,10 +20482,10 @@
         </is>
       </c>
       <c r="F376" t="n">
-        <v>37.61</v>
+        <v>108.76</v>
       </c>
       <c r="G376" t="n">
-        <v>44.38</v>
+        <v>128.34</v>
       </c>
       <c r="H376">
         <f>הגדרות!B8</f>
@@ -20505,165 +20505,6 @@
       </c>
       <c r="L376">
         <f>I376*(1+J376/100)+K376</f>
-        <v/>
-      </c>
-    </row>
-    <row r="377">
-      <c r="A377" t="inlineStr">
-        <is>
-          <t>פורינה (חנויות)</t>
-        </is>
-      </c>
-      <c r="B377" t="inlineStr">
-        <is>
-          <t>דוגלי בוגר בקר</t>
-        </is>
-      </c>
-      <c r="C377" t="inlineStr">
-        <is>
-          <t>חטיפים</t>
-        </is>
-      </c>
-      <c r="D377" t="inlineStr">
-        <is>
-          <t>12368766</t>
-        </is>
-      </c>
-      <c r="E377" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="F377" t="n">
-        <v>37.61</v>
-      </c>
-      <c r="G377" t="n">
-        <v>44.38</v>
-      </c>
-      <c r="H377">
-        <f>הגדרות!B8</f>
-        <v/>
-      </c>
-      <c r="I377">
-        <f>F377*(1-H377/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J377">
-        <f>הגדרות!C8</f>
-        <v/>
-      </c>
-      <c r="K377">
-        <f>הגדרות!D8</f>
-        <v/>
-      </c>
-      <c r="L377">
-        <f>I377*(1+J377/100)+K377</f>
-        <v/>
-      </c>
-    </row>
-    <row r="378">
-      <c r="A378" t="inlineStr">
-        <is>
-          <t>פורינה (חנויות)</t>
-        </is>
-      </c>
-      <c r="B378" t="inlineStr">
-        <is>
-          <t>דוגלי בוגר עוף</t>
-        </is>
-      </c>
-      <c r="C378" t="inlineStr">
-        <is>
-          <t>חטיפים</t>
-        </is>
-      </c>
-      <c r="D378" t="inlineStr">
-        <is>
-          <t>12368676</t>
-        </is>
-      </c>
-      <c r="E378" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="F378" t="n">
-        <v>108.76</v>
-      </c>
-      <c r="G378" t="n">
-        <v>128.34</v>
-      </c>
-      <c r="H378">
-        <f>הגדרות!B8</f>
-        <v/>
-      </c>
-      <c r="I378">
-        <f>F378*(1-H378/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J378">
-        <f>הגדרות!C8</f>
-        <v/>
-      </c>
-      <c r="K378">
-        <f>הגדרות!D8</f>
-        <v/>
-      </c>
-      <c r="L378">
-        <f>I378*(1+J378/100)+K378</f>
-        <v/>
-      </c>
-    </row>
-    <row r="379">
-      <c r="A379" t="inlineStr">
-        <is>
-          <t>פורינה (חנויות)</t>
-        </is>
-      </c>
-      <c r="B379" t="inlineStr">
-        <is>
-          <t>דוגלי בוגר בקר</t>
-        </is>
-      </c>
-      <c r="C379" t="inlineStr">
-        <is>
-          <t>חטיפים</t>
-        </is>
-      </c>
-      <c r="D379" t="inlineStr">
-        <is>
-          <t>12368675</t>
-        </is>
-      </c>
-      <c r="E379" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="F379" t="n">
-        <v>108.76</v>
-      </c>
-      <c r="G379" t="n">
-        <v>128.34</v>
-      </c>
-      <c r="H379">
-        <f>הגדרות!B8</f>
-        <v/>
-      </c>
-      <c r="I379">
-        <f>F379*(1-H379/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J379">
-        <f>הגדרות!C8</f>
-        <v/>
-      </c>
-      <c r="K379">
-        <f>הגדרות!D8</f>
-        <v/>
-      </c>
-      <c r="L379">
-        <f>I379*(1+J379/100)+K379</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
data(vetmarket): add the Invoices Plus store as a second confirmation source
Invoices Plus had 194 Vetmarket SKUs parsed from 05-08/2026 against the 171 published from
the vetmarket-cli store, and the two agree: 13 price differences across 116 shared SKUs, all
but one of them the newer month being higher. Merging on newest-month-wins adds 61 SKUs and
refreshes 32, 171 -> 232.

Only sku, description, list price and month are selected — discount_pct is the clinic's own
discount and is deliberately left behind. scripts/pull_invoices.sh makes the pull repeatable.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XoJGvA8cApVXFb92aBk3Fg
</commit_message>
<xml_diff>
--- a/downloads/shop.xlsx
+++ b/downloads/shop.xlsx
@@ -579,7 +579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L376"/>
+  <dimension ref="A1:L381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -16536,37 +16536,37 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>מדי-מרקט</t>
+          <t>וטמרקט</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>@ סדיניה 35 60X90 יח' TENA BED @</t>
+          <t>חטיף הילס היפואלרגני לכלב 200 גרם</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>אביזרים</t>
+          <t>חטיפים</t>
         </is>
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>33262-1</t>
+          <t>40608557</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="F302" t="n">
-        <v>31.36</v>
+        <v>24</v>
       </c>
       <c r="G302" t="n">
-        <v>37</v>
+        <v>28.32</v>
       </c>
       <c r="H302">
-        <f>הגדרות!B6</f>
+        <f>הגדרות!B5</f>
         <v/>
       </c>
       <c r="I302">
@@ -16574,11 +16574,11 @@
         <v/>
       </c>
       <c r="J302">
-        <f>הגדרות!C6</f>
+        <f>הגדרות!C5</f>
         <v/>
       </c>
       <c r="K302">
-        <f>הגדרות!D6</f>
+        <f>הגדרות!D5</f>
         <v/>
       </c>
       <c r="L302">
@@ -16589,37 +16589,37 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>מדי-מרקט</t>
+          <t>וטמרקט</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>ANTIGONE WIPES 19*20 500</t>
+          <t>חטיף ווג'ידנט Medium 15 יחידות, 352 גרם</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>חטיפים</t>
         </is>
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>M0002020</t>
+          <t>47307870</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="F303" t="n">
-        <v>71.42</v>
+        <v>24</v>
       </c>
       <c r="G303" t="n">
-        <v>84.27</v>
+        <v>28.32</v>
       </c>
       <c r="H303">
-        <f>הגדרות!B6</f>
+        <f>הגדרות!B5</f>
         <v/>
       </c>
       <c r="I303">
@@ -16627,11 +16627,11 @@
         <v/>
       </c>
       <c r="J303">
-        <f>הגדרות!C6</f>
+        <f>הגדרות!C5</f>
         <v/>
       </c>
       <c r="K303">
-        <f>הגדרות!D6</f>
+        <f>הגדרות!D5</f>
         <v/>
       </c>
       <c r="L303">
@@ -16642,37 +16642,37 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>מדי-מרקט</t>
+          <t>וטמרקט</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>ANTIGONE WIPES 20*20 200</t>
+          <t>חטיף פודיס מיני ענני עוף לחתולים, 50 גרם</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>חטיפים</t>
         </is>
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>100003</t>
+          <t>48000034</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="F304" t="n">
-        <v>30.32</v>
+        <v>3.5</v>
       </c>
       <c r="G304" t="n">
-        <v>35.78</v>
+        <v>4.13</v>
       </c>
       <c r="H304">
-        <f>הגדרות!B6</f>
+        <f>הגדרות!B5</f>
         <v/>
       </c>
       <c r="I304">
@@ -16680,11 +16680,11 @@
         <v/>
       </c>
       <c r="J304">
-        <f>הגדרות!C6</f>
+        <f>הגדרות!C5</f>
         <v/>
       </c>
       <c r="K304">
-        <f>הגדרות!D6</f>
+        <f>הגדרות!D5</f>
         <v/>
       </c>
       <c r="L304">
@@ -16695,37 +16695,37 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>מדי-מרקט</t>
+          <t>וטמרקט</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>CETRIN 1 LITTER SOL</t>
+          <t>חטיף פודיס מיני ענני ברווז לחתולים, 50 גרם</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>חול ושירותים</t>
+          <t>חטיפים</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>33365</t>
+          <t>48000035</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="F305" t="n">
-        <v>30.84</v>
+        <v>3.5</v>
       </c>
       <c r="G305" t="n">
-        <v>36.39</v>
+        <v>4.13</v>
       </c>
       <c r="H305">
-        <f>הגדרות!B6</f>
+        <f>הגדרות!B5</f>
         <v/>
       </c>
       <c r="I305">
@@ -16733,11 +16733,11 @@
         <v/>
       </c>
       <c r="J305">
-        <f>הגדרות!C6</f>
+        <f>הגדרות!C5</f>
         <v/>
       </c>
       <c r="K305">
-        <f>הגדרות!D6</f>
+        <f>הגדרות!D5</f>
         <v/>
       </c>
       <c r="L305">
@@ -16748,37 +16748,37 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>מדי-מרקט</t>
+          <t>וטמרקט</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>DOUXO S3 CALM MOUSSE 150 ML</t>
+          <t>חטיף פודיס דגיגוני סלמון לחתולים, 50 גרם</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>חטיפים</t>
         </is>
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>81-105</t>
+          <t>48000036</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="F306" t="n">
-        <v>58.47</v>
+        <v>3.5</v>
       </c>
       <c r="G306" t="n">
-        <v>69</v>
+        <v>4.13</v>
       </c>
       <c r="H306">
-        <f>הגדרות!B6</f>
+        <f>הגדרות!B5</f>
         <v/>
       </c>
       <c r="I306">
@@ -16786,11 +16786,11 @@
         <v/>
       </c>
       <c r="J306">
-        <f>הגדרות!C6</f>
+        <f>הגדרות!C5</f>
         <v/>
       </c>
       <c r="K306">
-        <f>הגדרות!D6</f>
+        <f>הגדרות!D5</f>
         <v/>
       </c>
       <c r="L306">
@@ -16806,17 +16806,17 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>DOUXO S3 PYO MOUSSE 150 ML</t>
+          <t>@ סדיניה 35 60X90 יח' TENA BED @</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>אביזרים</t>
         </is>
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>81-101</t>
+          <t>33262-1</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -16825,10 +16825,10 @@
         </is>
       </c>
       <c r="F307" t="n">
-        <v>58.47</v>
+        <v>31.36</v>
       </c>
       <c r="G307" t="n">
-        <v>69</v>
+        <v>37</v>
       </c>
       <c r="H307">
         <f>הגדרות!B6</f>
@@ -16859,7 +16859,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>DOUXO S3 PYO PADS</t>
+          <t>ANTIGONE WIPES 19*20 500</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -16869,7 +16869,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>81-107</t>
+          <t>M0002020</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -16878,10 +16878,10 @@
         </is>
       </c>
       <c r="F308" t="n">
-        <v>36.44</v>
+        <v>71.42</v>
       </c>
       <c r="G308" t="n">
-        <v>43</v>
+        <v>84.27</v>
       </c>
       <c r="H308">
         <f>הגדרות!B6</f>
@@ -16912,7 +16912,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>DOUXO S3 SEB MOUSSE 150 ML</t>
+          <t>ANTIGONE WIPES 20*20 200</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -16922,7 +16922,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>81-103</t>
+          <t>100003</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
@@ -16931,10 +16931,10 @@
         </is>
       </c>
       <c r="F309" t="n">
-        <v>58.47</v>
+        <v>30.32</v>
       </c>
       <c r="G309" t="n">
-        <v>69</v>
+        <v>35.78</v>
       </c>
       <c r="H309">
         <f>הגדרות!B6</f>
@@ -16965,7 +16965,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Easy Go 500 Litter - איזי גו</t>
+          <t>CETRIN 1 LITTER SOL</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -16975,7 +16975,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>18033-1</t>
+          <t>33365</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -16984,10 +16984,10 @@
         </is>
       </c>
       <c r="F310" t="n">
-        <v>14.32</v>
+        <v>30.84</v>
       </c>
       <c r="G310" t="n">
-        <v>16.9</v>
+        <v>36.39</v>
       </c>
       <c r="H310">
         <f>הגדרות!B6</f>
@@ -17018,17 +17018,17 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Pinchers 45chews peanut butter pill hiding treat</t>
+          <t>DOUXO S3 CALM MOUSSE 150 ML</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>חטיפים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>090062J.045</t>
+          <t>81-105</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -17037,10 +17037,10 @@
         </is>
       </c>
       <c r="F311" t="n">
-        <v>22.3</v>
+        <v>58.47</v>
       </c>
       <c r="G311" t="n">
-        <v>26.31</v>
+        <v>69</v>
       </c>
       <c r="H311">
         <f>הגדרות!B6</f>
@@ -17071,17 +17071,17 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>אלונקה רכה מתקפלת NAR QuikLitter</t>
+          <t>DOUXO S3 PYO MOUSSE 150 ML</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>חול ושירותים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>4105</t>
+          <t>81-101</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -17090,10 +17090,10 @@
         </is>
       </c>
       <c r="F312" t="n">
-        <v>194.49</v>
+        <v>58.47</v>
       </c>
       <c r="G312" t="n">
-        <v>229.5</v>
+        <v>69</v>
       </c>
       <c r="H312">
         <f>הגדרות!B6</f>
@@ -17124,7 +17124,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>כלוב נשיאה אטלס 10 ללא מזרון Ferplast</t>
+          <t>DOUXO S3 PYO PADS</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -17134,7 +17134,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>5550279</t>
+          <t>81-107</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -17143,10 +17143,10 @@
         </is>
       </c>
       <c r="F313" t="n">
-        <v>50.85</v>
+        <v>36.44</v>
       </c>
       <c r="G313" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="H313">
         <f>הגדרות!B6</f>
@@ -17177,7 +17177,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>כלוב נשיאה אטלס 20 ללא מזרון Ferplast</t>
+          <t>DOUXO S3 SEB MOUSSE 150 ML</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -17187,7 +17187,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>5550280</t>
+          <t>81-103</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -17196,10 +17196,10 @@
         </is>
       </c>
       <c r="F314" t="n">
-        <v>88.14</v>
+        <v>58.47</v>
       </c>
       <c r="G314" t="n">
-        <v>104</v>
+        <v>69</v>
       </c>
       <c r="H314">
         <f>הגדרות!B6</f>
@@ -17230,17 +17230,17 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>מברשת רחצת ידיים לפני ניתוח, סטר', מדיקפרו</t>
+          <t>Easy Go 500 Litter - איזי גו</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>חול ושירותים</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>3694</t>
+          <t>18033-1</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -17249,10 +17249,10 @@
         </is>
       </c>
       <c r="F315" t="n">
-        <v>0.87</v>
+        <v>14.32</v>
       </c>
       <c r="G315" t="n">
-        <v>1.03</v>
+        <v>16.9</v>
       </c>
       <c r="H315">
         <f>הגדרות!B6</f>
@@ -17283,17 +17283,17 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>מגבונים - Clinell sporicidal wipesn 1/6</t>
+          <t>Pinchers 45chews peanut butter pill hiding treat</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>חטיפים</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>CS25</t>
+          <t>090062J.045</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -17302,10 +17302,10 @@
         </is>
       </c>
       <c r="F316" t="n">
-        <v>156.78</v>
+        <v>22.3</v>
       </c>
       <c r="G316" t="n">
-        <v>185</v>
+        <v>26.31</v>
       </c>
       <c r="H316">
         <f>הגדרות!B6</f>
@@ -17336,17 +17336,17 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>מגבונים - Clinell Universal wipes clip pack 50</t>
+          <t>אלונקה רכה מתקפלת NAR QuikLitter</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>חול ושירותים</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>11050</t>
+          <t>4105</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -17355,10 +17355,10 @@
         </is>
       </c>
       <c r="F317" t="n">
-        <v>9.25</v>
+        <v>194.49</v>
       </c>
       <c r="G317" t="n">
-        <v>10.92</v>
+        <v>229.5</v>
       </c>
       <c r="H317">
         <f>הגדרות!B6</f>
@@ -17389,7 +17389,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>מגבונים - Clinell Universal Wipes pack of 200</t>
+          <t>כלוב נשיאה אטלס 10 ללא מזרון Ferplast</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -17399,7 +17399,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>11200</t>
+          <t>5550279</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -17408,10 +17408,10 @@
         </is>
       </c>
       <c r="F318" t="n">
-        <v>19.92</v>
+        <v>50.85</v>
       </c>
       <c r="G318" t="n">
-        <v>23.5</v>
+        <v>60</v>
       </c>
       <c r="H318">
         <f>הגדרות!B6</f>
@@ -17442,7 +17442,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>מגבונים מדי-קלין אקסטרה עבים מועשר באלוורה 500 יח 20X16 ס"מ</t>
+          <t>כלוב נשיאה אטלס 20 ללא מזרון Ferplast</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -17452,7 +17452,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>128697</t>
+          <t>5550280</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -17461,10 +17461,10 @@
         </is>
       </c>
       <c r="F319" t="n">
-        <v>22.88</v>
+        <v>88.14</v>
       </c>
       <c r="G319" t="n">
-        <v>27</v>
+        <v>104</v>
       </c>
       <c r="H319">
         <f>הגדרות!B6</f>
@@ -17495,7 +17495,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>מגבונים מדי-קלין מועשרים באלוורה 500 יח' 28X20 ס"מ</t>
+          <t>מברשת רחצת ידיים לפני ניתוח, סטר', מדיקפרו</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -17505,7 +17505,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>128695</t>
+          <t>3694</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -17514,10 +17514,10 @@
         </is>
       </c>
       <c r="F320" t="n">
-        <v>22.88</v>
+        <v>0.87</v>
       </c>
       <c r="G320" t="n">
-        <v>27</v>
+        <v>1.03</v>
       </c>
       <c r="H320">
         <f>הגדרות!B6</f>
@@ -17548,17 +17548,17 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>מיטה חשמלית דגם GUESS 402 מעקה מגלוון</t>
+          <t>מגבונים - Clinell sporicidal wipesn 1/6</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>אביזרים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>883135</t>
+          <t>CS25</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -17567,10 +17567,10 @@
         </is>
       </c>
       <c r="F321" t="n">
-        <v>6288.14</v>
+        <v>156.78</v>
       </c>
       <c r="G321" t="n">
-        <v>7420</v>
+        <v>185</v>
       </c>
       <c r="H321">
         <f>הגדרות!B6</f>
@@ -17601,7 +17601,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>מספריים אל חלד לציפורניים REISZ</t>
+          <t>מגבונים - Clinell Universal wipes clip pack 50</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -17611,7 +17611,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>434457</t>
+          <t>11050</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -17620,10 +17620,10 @@
         </is>
       </c>
       <c r="F322" t="n">
-        <v>21.17</v>
+        <v>9.25</v>
       </c>
       <c r="G322" t="n">
-        <v>24.98</v>
+        <v>10.92</v>
       </c>
       <c r="H322">
         <f>הגדרות!B6</f>
@@ -17654,7 +17654,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>משושת ג'ל 500 מ"ל פוליגונום רב תכליתי Herbaderm</t>
+          <t>מגבונים - Clinell Universal Wipes pack of 200</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -17664,7 +17664,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>67-105</t>
+          <t>11200</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -17673,10 +17673,10 @@
         </is>
       </c>
       <c r="F323" t="n">
-        <v>157.63</v>
+        <v>19.92</v>
       </c>
       <c r="G323" t="n">
-        <v>186</v>
+        <v>23.5</v>
       </c>
       <c r="H323">
         <f>הגדרות!B6</f>
@@ -17707,7 +17707,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>משושת קרם 500 מ"ל פוליגונום רב תכליתי Herbaderm</t>
+          <t>מגבונים מדי-קלין אקסטרה עבים מועשר באלוורה 500 יח 20X16 ס"מ</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -17717,7 +17717,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>67-103</t>
+          <t>128697</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -17726,10 +17726,10 @@
         </is>
       </c>
       <c r="F324" t="n">
-        <v>157.63</v>
+        <v>22.88</v>
       </c>
       <c r="G324" t="n">
-        <v>186</v>
+        <v>27</v>
       </c>
       <c r="H324">
         <f>הגדרות!B6</f>
@@ -17760,7 +17760,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>נייר לניגוב עדשות מיקרוסקופ 1159 1/280 Kimwipes</t>
+          <t>מגבונים מדי-קלין מועשרים באלוורה 500 יח' 28X20 ס"מ</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -17770,7 +17770,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>3422</t>
+          <t>128695</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -17779,10 +17779,10 @@
         </is>
       </c>
       <c r="F325" t="n">
-        <v>26.44</v>
+        <v>22.88</v>
       </c>
       <c r="G325" t="n">
-        <v>31.2</v>
+        <v>27</v>
       </c>
       <c r="H325">
         <f>הגדרות!B6</f>
@@ -17813,7 +17813,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>סיר לילה פלסטיק/ מיטה גדול עם ידית, מדיקפרו</t>
+          <t>מיטה חשמלית דגם GUESS 402 מעקה מגלוון</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -17823,7 +17823,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>4055</t>
+          <t>883135</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -17832,10 +17832,10 @@
         </is>
       </c>
       <c r="F326" t="n">
-        <v>11.86</v>
+        <v>6288.14</v>
       </c>
       <c r="G326" t="n">
-        <v>14</v>
+        <v>7420</v>
       </c>
       <c r="H326">
         <f>הגדרות!B6</f>
@@ -17866,7 +17866,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>קוצץ ציפורניים, מדיקפרו</t>
+          <t>מספריים אל חלד לציפורניים REISZ</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -17876,7 +17876,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>17709</t>
+          <t>434457</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -17885,10 +17885,10 @@
         </is>
       </c>
       <c r="F327" t="n">
-        <v>3.32</v>
+        <v>21.17</v>
       </c>
       <c r="G327" t="n">
-        <v>3.92</v>
+        <v>24.98</v>
       </c>
       <c r="H327">
         <f>הגדרות!B6</f>
@@ -17919,7 +17919,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>ראש למכונת תספורת (סכין) 40 - 0.25 מ"מ LAUBE</t>
+          <t>משושת ג'ל 500 מ"ל פוליגונום רב תכליתי Herbaderm</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -17929,7 +17929,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>80662</t>
+          <t>67-105</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -17938,10 +17938,10 @@
         </is>
       </c>
       <c r="F328" t="n">
-        <v>120.13</v>
+        <v>157.63</v>
       </c>
       <c r="G328" t="n">
-        <v>141.75</v>
+        <v>186</v>
       </c>
       <c r="H328">
         <f>הגדרות!B6</f>
@@ -17972,17 +17972,17 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>רצועה ללוח גב צבע כתום עם אבזם מתכת</t>
+          <t>משושת קרם 500 מ"ל פוליגונום רב תכליתי Herbaderm</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>אביזרים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>16155</t>
+          <t>67-103</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -17991,10 +17991,10 @@
         </is>
       </c>
       <c r="F329" t="n">
-        <v>71.19</v>
+        <v>157.63</v>
       </c>
       <c r="G329" t="n">
-        <v>84</v>
+        <v>186</v>
       </c>
       <c r="H329">
         <f>הגדרות!B6</f>
@@ -18025,17 +18025,17 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>רצועה לתמיכה למסכת טרכוסטומי L</t>
+          <t>נייר לניגוב עדשות מיקרוסקופ 1159 1/280 Kimwipes</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>אביזרים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>7985</t>
+          <t>3422</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -18044,10 +18044,10 @@
         </is>
       </c>
       <c r="F330" t="n">
-        <v>5.91</v>
+        <v>26.44</v>
       </c>
       <c r="G330" t="n">
-        <v>6.97</v>
+        <v>31.2</v>
       </c>
       <c r="H330">
         <f>הגדרות!B6</f>
@@ -18078,7 +18078,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>רצועה לתמיכה למסכת טרכוסטומי M</t>
+          <t>סיר לילה פלסטיק/ מיטה גדול עם ידית, מדיקפרו</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -18088,7 +18088,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>7987</t>
+          <t>4055</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -18097,10 +18097,10 @@
         </is>
       </c>
       <c r="F331" t="n">
-        <v>6.19</v>
+        <v>11.86</v>
       </c>
       <c r="G331" t="n">
-        <v>7.3</v>
+        <v>14</v>
       </c>
       <c r="H331">
         <f>הגדרות!B6</f>
@@ -18131,17 +18131,17 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>רצועה לתמיכה למסכת טרכוסטומי XL</t>
+          <t>קוצץ ציפורניים, מדיקפרו</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>אביזרים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>7986</t>
+          <t>17709</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -18150,10 +18150,10 @@
         </is>
       </c>
       <c r="F332" t="n">
-        <v>6.36</v>
+        <v>3.32</v>
       </c>
       <c r="G332" t="n">
-        <v>7.5</v>
+        <v>3.92</v>
       </c>
       <c r="H332">
         <f>הגדרות!B6</f>
@@ -18179,12 +18179,12 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>פט-וט ביומד</t>
+          <t>מדי-מרקט</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Keto Tris Finger Wipes 50 units</t>
+          <t>ראש למכונת תספורת (סכין) 40 - 0.25 מ"מ LAUBE</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -18194,22 +18194,22 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>DERMA-SP1330</t>
+          <t>80662</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F333" t="n">
-        <v>59</v>
+        <v>120.13</v>
       </c>
       <c r="G333" t="n">
-        <v>69.62</v>
+        <v>141.75</v>
       </c>
       <c r="H333">
-        <f>הגדרות!B7</f>
+        <f>הגדרות!B6</f>
         <v/>
       </c>
       <c r="I333">
@@ -18217,11 +18217,11 @@
         <v/>
       </c>
       <c r="J333">
-        <f>הגדרות!C7</f>
+        <f>הגדרות!C6</f>
         <v/>
       </c>
       <c r="K333">
-        <f>הגדרות!D7</f>
+        <f>הגדרות!D6</f>
         <v/>
       </c>
       <c r="L333">
@@ -18232,37 +18232,37 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>פט-וט ביומד</t>
+          <t>מדי-מרקט</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Tris Ophto Wipes 50ct</t>
+          <t>רצועה ללוח גב צבע כתום עם אבזם מתכת</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>אביזרים</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>DZOO-TWX</t>
+          <t>16155</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F334" t="n">
-        <v>58</v>
+        <v>71.19</v>
       </c>
       <c r="G334" t="n">
-        <v>68.44</v>
+        <v>84</v>
       </c>
       <c r="H334">
-        <f>הגדרות!B7</f>
+        <f>הגדרות!B6</f>
         <v/>
       </c>
       <c r="I334">
@@ -18270,11 +18270,11 @@
         <v/>
       </c>
       <c r="J334">
-        <f>הגדרות!C7</f>
+        <f>הגדרות!C6</f>
         <v/>
       </c>
       <c r="K334">
-        <f>הגדרות!D7</f>
+        <f>הגדרות!D6</f>
         <v/>
       </c>
       <c r="L334">
@@ -18285,37 +18285,37 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>פט-וט ביומד</t>
+          <t>מדי-מרקט</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Pill Splitter</t>
+          <t>רצועה לתמיכה למסכת טרכוסטומי L</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>חול ושירותים</t>
+          <t>אביזרים</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>FIONA-821070-1</t>
+          <t>7985</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F335" t="n">
-        <v>7</v>
+        <v>5.91</v>
       </c>
       <c r="G335" t="n">
-        <v>8.26</v>
+        <v>6.97</v>
       </c>
       <c r="H335">
-        <f>הגדרות!B7</f>
+        <f>הגדרות!B6</f>
         <v/>
       </c>
       <c r="I335">
@@ -18323,11 +18323,11 @@
         <v/>
       </c>
       <c r="J335">
-        <f>הגדרות!C7</f>
+        <f>הגדרות!C6</f>
         <v/>
       </c>
       <c r="K335">
-        <f>הגדרות!D7</f>
+        <f>הגדרות!D6</f>
         <v/>
       </c>
       <c r="L335">
@@ -18338,37 +18338,37 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>פט-וט ביומד</t>
+          <t>מדי-מרקט</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Calming Spray 200ml</t>
+          <t>רצועה לתמיכה למסכת טרכוסטומי M</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>הרגעה</t>
+          <t>אביזרים</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>PR-79583</t>
+          <t>7987</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F336" t="n">
-        <v>46</v>
+        <v>6.19</v>
       </c>
       <c r="G336" t="n">
-        <v>54.28</v>
+        <v>7.3</v>
       </c>
       <c r="H336">
-        <f>הגדרות!B7</f>
+        <f>הגדרות!B6</f>
         <v/>
       </c>
       <c r="I336">
@@ -18376,11 +18376,11 @@
         <v/>
       </c>
       <c r="J336">
-        <f>הגדרות!C7</f>
+        <f>הגדרות!C6</f>
         <v/>
       </c>
       <c r="K336">
-        <f>הגדרות!D7</f>
+        <f>הגדרות!D6</f>
         <v/>
       </c>
       <c r="L336">
@@ -18391,37 +18391,37 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>פט-וט ביומד</t>
+          <t>מדי-מרקט</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Mini Calming Spray 15ml</t>
+          <t>רצועה לתמיכה למסכת טרכוסטומי XL</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>הרגעה</t>
+          <t>אביזרים</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>PR-79664</t>
+          <t>7986</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F337" t="n">
-        <v>18</v>
+        <v>6.36</v>
       </c>
       <c r="G337" t="n">
-        <v>21.24</v>
+        <v>7.5</v>
       </c>
       <c r="H337">
-        <f>הגדרות!B7</f>
+        <f>הגדרות!B6</f>
         <v/>
       </c>
       <c r="I337">
@@ -18429,11 +18429,11 @@
         <v/>
       </c>
       <c r="J337">
-        <f>הגדרות!C7</f>
+        <f>הגדרות!C6</f>
         <v/>
       </c>
       <c r="K337">
-        <f>הגדרות!D7</f>
+        <f>הגדרות!D6</f>
         <v/>
       </c>
       <c r="L337">
@@ -18449,17 +18449,17 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Battery Atomizer Refill 300ml</t>
+          <t>Keto Tris Finger Wipes 50 units</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>הרגעה</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>PR-79744</t>
+          <t>DERMA-SP1330</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
@@ -18468,10 +18468,10 @@
         </is>
       </c>
       <c r="F338" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G338" t="n">
-        <v>66.08</v>
+        <v>69.62</v>
       </c>
       <c r="H338">
         <f>הגדרות!B7</f>
@@ -18502,17 +18502,17 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Battery Atomizer</t>
+          <t>Tris Ophto Wipes 50ct</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>הרגעה</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>PR-79745</t>
+          <t>DZOO-TWX</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -18521,10 +18521,10 @@
         </is>
       </c>
       <c r="F339" t="n">
-        <v>185</v>
+        <v>58</v>
       </c>
       <c r="G339" t="n">
-        <v>218.3</v>
+        <v>68.44</v>
       </c>
       <c r="H339">
         <f>הגדרות!B7</f>
@@ -18555,17 +18555,17 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Calming Wipe Sachet (12)</t>
+          <t>Pill Splitter</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>הרגעה</t>
+          <t>חול ושירותים</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>PR-79881</t>
+          <t>FIONA-821070-1</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
@@ -18574,10 +18574,10 @@
         </is>
       </c>
       <c r="F340" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="G340" t="n">
-        <v>21.24</v>
+        <v>8.26</v>
       </c>
       <c r="H340">
         <f>הגדרות!B7</f>
@@ -18608,17 +18608,17 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Boredom Buster forager kit</t>
+          <t>Calming Spray 200ml</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>צעצועים</t>
+          <t>הרגעה</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>PR-80128</t>
+          <t>PR-79583</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
@@ -18627,10 +18627,10 @@
         </is>
       </c>
       <c r="F341" t="n">
-        <v>105</v>
+        <v>46</v>
       </c>
       <c r="G341" t="n">
-        <v>123.9</v>
+        <v>54.28</v>
       </c>
       <c r="H341">
         <f>הגדרות!B7</f>
@@ -18661,7 +18661,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Calming Bandana Kit EXTRA SMALL</t>
+          <t>Mini Calming Spray 15ml</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -18671,7 +18671,7 @@
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>PR-79959</t>
+          <t>PR-79664</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
@@ -18680,10 +18680,10 @@
         </is>
       </c>
       <c r="F342" t="n">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="G342" t="n">
-        <v>51.92</v>
+        <v>21.24</v>
       </c>
       <c r="H342">
         <f>הגדרות!B7</f>
@@ -18714,7 +18714,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Calming Bandana Kit SMALL</t>
+          <t>Battery Atomizer Refill 300ml</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -18724,7 +18724,7 @@
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>PR-79960</t>
+          <t>PR-79744</t>
         </is>
       </c>
       <c r="E343" t="inlineStr">
@@ -18733,10 +18733,10 @@
         </is>
       </c>
       <c r="F343" t="n">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="G343" t="n">
-        <v>51.92</v>
+        <v>66.08</v>
       </c>
       <c r="H343">
         <f>הגדרות!B7</f>
@@ -18767,7 +18767,7 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Calming Bandana Kit MEDIUM</t>
+          <t>Battery Atomizer</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
@@ -18777,7 +18777,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>PR-79961</t>
+          <t>PR-79745</t>
         </is>
       </c>
       <c r="E344" t="inlineStr">
@@ -18786,10 +18786,10 @@
         </is>
       </c>
       <c r="F344" t="n">
-        <v>44</v>
+        <v>185</v>
       </c>
       <c r="G344" t="n">
-        <v>51.92</v>
+        <v>218.3</v>
       </c>
       <c r="H344">
         <f>הגדרות!B7</f>
@@ -18820,7 +18820,7 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Calming Bandana Kit LARGE</t>
+          <t>Calming Wipe Sachet (12)</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -18830,7 +18830,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>PR-79962</t>
+          <t>PR-79881</t>
         </is>
       </c>
       <c r="E345" t="inlineStr">
@@ -18839,10 +18839,10 @@
         </is>
       </c>
       <c r="F345" t="n">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="G345" t="n">
-        <v>51.92</v>
+        <v>21.24</v>
       </c>
       <c r="H345">
         <f>הגדרות!B7</f>
@@ -18873,17 +18873,17 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Calming Spray 400ml – PROF. PACK</t>
+          <t>Boredom Buster forager kit</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>הרגעה</t>
+          <t>צעצועים</t>
         </is>
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>PR-79983</t>
+          <t>PR-80128</t>
         </is>
       </c>
       <c r="E346" t="inlineStr">
@@ -18892,10 +18892,10 @@
         </is>
       </c>
       <c r="F346" t="n">
-        <v>61</v>
+        <v>105</v>
       </c>
       <c r="G346" t="n">
-        <v>71.98</v>
+        <v>123.9</v>
       </c>
       <c r="H346">
         <f>הגדרות!B7</f>
@@ -18921,37 +18921,37 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>פורינה (חנויות)</t>
+          <t>פט-וט ביומד</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס אוריגי'נל קראנץ</t>
+          <t>Calming Bandana Kit EXTRA SMALL</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>חטיפים</t>
+          <t>הרגעה</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>12348261</t>
+          <t>PR-79959</t>
         </is>
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="F347" t="n">
-        <v>8.18</v>
+        <v>44</v>
       </c>
       <c r="G347" t="n">
-        <v>9.65</v>
+        <v>51.92</v>
       </c>
       <c r="H347">
-        <f>הגדרות!B8</f>
+        <f>הגדרות!B7</f>
         <v/>
       </c>
       <c r="I347">
@@ -18959,11 +18959,11 @@
         <v/>
       </c>
       <c r="J347">
-        <f>הגדרות!C8</f>
+        <f>הגדרות!C7</f>
         <v/>
       </c>
       <c r="K347">
-        <f>הגדרות!D8</f>
+        <f>הגדרות!D7</f>
         <v/>
       </c>
       <c r="L347">
@@ -18974,37 +18974,37 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>פורינה (חנויות)</t>
+          <t>פט-וט ביומד</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס מיקס גריל קראנץ</t>
+          <t>Calming Bandana Kit SMALL</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>חטיפים</t>
+          <t>הרגעה</t>
         </is>
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>12348037</t>
+          <t>PR-79960</t>
         </is>
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="F348" t="n">
-        <v>8.18</v>
+        <v>44</v>
       </c>
       <c r="G348" t="n">
-        <v>9.65</v>
+        <v>51.92</v>
       </c>
       <c r="H348">
-        <f>הגדרות!B8</f>
+        <f>הגדרות!B7</f>
         <v/>
       </c>
       <c r="I348">
@@ -19012,11 +19012,11 @@
         <v/>
       </c>
       <c r="J348">
-        <f>הגדרות!C8</f>
+        <f>הגדרות!C7</f>
         <v/>
       </c>
       <c r="K348">
-        <f>הגדרות!D8</f>
+        <f>הגדרות!D7</f>
         <v/>
       </c>
       <c r="L348">
@@ -19027,37 +19027,37 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>פורינה (חנויות)</t>
+          <t>פט-וט ביומד</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס מעדני ים קראנץ</t>
+          <t>Calming Bandana Kit MEDIUM</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>חטיפים</t>
+          <t>הרגעה</t>
         </is>
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>12364507</t>
+          <t>PR-79961</t>
         </is>
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="F349" t="n">
-        <v>8.18</v>
+        <v>44</v>
       </c>
       <c r="G349" t="n">
-        <v>9.65</v>
+        <v>51.92</v>
       </c>
       <c r="H349">
-        <f>הגדרות!B8</f>
+        <f>הגדרות!B7</f>
         <v/>
       </c>
       <c r="I349">
@@ -19065,11 +19065,11 @@
         <v/>
       </c>
       <c r="J349">
-        <f>הגדרות!C8</f>
+        <f>הגדרות!C7</f>
         <v/>
       </c>
       <c r="K349">
-        <f>הגדרות!D8</f>
+        <f>הגדרות!D7</f>
         <v/>
       </c>
       <c r="L349">
@@ -19080,37 +19080,37 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>פורינה (חנויות)</t>
+          <t>פט-וט ביומד</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס פיקניק קרנץ</t>
+          <t>Calming Bandana Kit LARGE</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>חטיפים</t>
+          <t>הרגעה</t>
         </is>
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>12368621</t>
+          <t>PR-79962</t>
         </is>
       </c>
       <c r="E350" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="F350" t="n">
-        <v>8.18</v>
+        <v>44</v>
       </c>
       <c r="G350" t="n">
-        <v>9.65</v>
+        <v>51.92</v>
       </c>
       <c r="H350">
-        <f>הגדרות!B8</f>
+        <f>הגדרות!B7</f>
         <v/>
       </c>
       <c r="I350">
@@ -19118,11 +19118,11 @@
         <v/>
       </c>
       <c r="J350">
-        <f>הגדרות!C8</f>
+        <f>הגדרות!C7</f>
         <v/>
       </c>
       <c r="K350">
-        <f>הגדרות!D8</f>
+        <f>הגדרות!D7</f>
         <v/>
       </c>
       <c r="L350">
@@ -19133,37 +19133,37 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>פורינה (חנויות)</t>
+          <t>פט-וט ביומד</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס קרייזי צ'יז</t>
+          <t>Calming Spray 400ml – PROF. PACK</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>חטיפים</t>
+          <t>הרגעה</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>12528489</t>
+          <t>PR-79983</t>
         </is>
       </c>
       <c r="E351" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="F351" t="n">
-        <v>8.18</v>
+        <v>61</v>
       </c>
       <c r="G351" t="n">
-        <v>9.65</v>
+        <v>71.98</v>
       </c>
       <c r="H351">
-        <f>הגדרות!B8</f>
+        <f>הגדרות!B7</f>
         <v/>
       </c>
       <c r="I351">
@@ -19171,11 +19171,11 @@
         <v/>
       </c>
       <c r="J351">
-        <f>הגדרות!C8</f>
+        <f>הגדרות!C7</f>
         <v/>
       </c>
       <c r="K351">
-        <f>הגדרות!D8</f>
+        <f>הגדרות!D7</f>
         <v/>
       </c>
       <c r="L351">
@@ -19191,7 +19191,7 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס מאנץ' בוקר</t>
+          <t>פריסקיז פארטי מיקס אוריגי'נל קראנץ</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -19201,7 +19201,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>12280472</t>
+          <t>12348261</t>
         </is>
       </c>
       <c r="E352" t="inlineStr">
@@ -19244,7 +19244,7 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס הודו</t>
+          <t>פריסקיז פארטי מיקס מיקס גריל קראנץ</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -19254,7 +19254,7 @@
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>12332654</t>
+          <t>12348037</t>
         </is>
       </c>
       <c r="E353" t="inlineStr">
@@ -19297,7 +19297,7 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס עוף</t>
+          <t>פריסקיז פארטי מיקס מעדני ים קראנץ</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -19307,7 +19307,7 @@
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>12332617</t>
+          <t>12364507</t>
         </is>
       </c>
       <c r="E354" t="inlineStr">
@@ -19350,7 +19350,7 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>פריסקיז פלייפולס סלמון ושרימפס</t>
+          <t>פריסקיז פארטי מיקס פיקניק קרנץ</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -19360,7 +19360,7 @@
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>12534203</t>
+          <t>12368621</t>
         </is>
       </c>
       <c r="E355" t="inlineStr">
@@ -19403,7 +19403,7 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>פריסקיז פלייפולס עוף וכבד</t>
+          <t>פריסקיז פארטי מיקס קרייזי צ'יז</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -19413,7 +19413,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>12534194</t>
+          <t>12528489</t>
         </is>
       </c>
       <c r="E356" t="inlineStr">
@@ -19456,7 +19456,7 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>פריסקיז צנצנת פארטי מיקס מעדני ים קראנץ</t>
+          <t>פריסקיז פארטי מיקס מאנץ' בוקר</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -19466,7 +19466,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>12364794</t>
+          <t>12280472</t>
         </is>
       </c>
       <c r="E357" t="inlineStr">
@@ -19475,10 +19475,10 @@
         </is>
       </c>
       <c r="F357" t="n">
-        <v>50.67</v>
+        <v>8.18</v>
       </c>
       <c r="G357" t="n">
-        <v>59.79</v>
+        <v>9.65</v>
       </c>
       <c r="H357">
         <f>הגדרות!B8</f>
@@ -19509,7 +19509,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>פריסקיז צנצנת פארטי מיקס אוריגי'נל קראנץ</t>
+          <t>פריסקיז פארטי מיקס הודו</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -19519,7 +19519,7 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>12349730</t>
+          <t>12332654</t>
         </is>
       </c>
       <c r="E358" t="inlineStr">
@@ -19528,10 +19528,10 @@
         </is>
       </c>
       <c r="F358" t="n">
-        <v>50.67</v>
+        <v>8.18</v>
       </c>
       <c r="G358" t="n">
-        <v>59.79</v>
+        <v>9.65</v>
       </c>
       <c r="H358">
         <f>הגדרות!B8</f>
@@ -19562,7 +19562,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>דנטלייף לכלב מגזע קטן</t>
+          <t>פריסקיז פארטי מיקס עוף</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -19572,7 +19572,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>12606950</t>
+          <t>12332617</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
@@ -19581,10 +19581,10 @@
         </is>
       </c>
       <c r="F359" t="n">
-        <v>10.2</v>
+        <v>8.18</v>
       </c>
       <c r="G359" t="n">
-        <v>12.04</v>
+        <v>9.65</v>
       </c>
       <c r="H359">
         <f>הגדרות!B8</f>
@@ -19615,7 +19615,7 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>דנטלייף לכלב מגזע בינוני</t>
+          <t>פריסקיז פלייפולס סלמון ושרימפס</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -19625,7 +19625,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>12606926</t>
+          <t>12534203</t>
         </is>
       </c>
       <c r="E360" t="inlineStr">
@@ -19634,10 +19634,10 @@
         </is>
       </c>
       <c r="F360" t="n">
-        <v>10.2</v>
+        <v>8.18</v>
       </c>
       <c r="G360" t="n">
-        <v>12.04</v>
+        <v>9.65</v>
       </c>
       <c r="H360">
         <f>הגדרות!B8</f>
@@ -19668,7 +19668,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>דנטלייף לכלב מגזע גדול</t>
+          <t>פריסקיז פלייפולס עוף וכבד</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -19678,7 +19678,7 @@
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>12606948</t>
+          <t>12534194</t>
         </is>
       </c>
       <c r="E361" t="inlineStr">
@@ -19687,10 +19687,10 @@
         </is>
       </c>
       <c r="F361" t="n">
-        <v>10.2</v>
+        <v>8.18</v>
       </c>
       <c r="G361" t="n">
-        <v>12.04</v>
+        <v>9.65</v>
       </c>
       <c r="H361">
         <f>הגדרות!B8</f>
@@ -19721,7 +19721,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>דנטלייף חתול עוף</t>
+          <t>פריסקיז צנצנת פארטי מיקס מעדני ים קראנץ</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -19731,7 +19731,7 @@
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>12607325</t>
+          <t>12364794</t>
         </is>
       </c>
       <c r="E362" t="inlineStr">
@@ -19740,10 +19740,10 @@
         </is>
       </c>
       <c r="F362" t="n">
-        <v>6.5</v>
+        <v>50.67</v>
       </c>
       <c r="G362" t="n">
-        <v>7.67</v>
+        <v>59.79</v>
       </c>
       <c r="H362">
         <f>הגדרות!B8</f>
@@ -19774,7 +19774,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>דנטלייף חתול סלמון</t>
+          <t>פריסקיז צנצנת פארטי מיקס אוריגי'נל קראנץ</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -19784,7 +19784,7 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>12607342</t>
+          <t>12349730</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
@@ -19793,10 +19793,10 @@
         </is>
       </c>
       <c r="F363" t="n">
-        <v>6.5</v>
+        <v>50.67</v>
       </c>
       <c r="G363" t="n">
-        <v>7.67</v>
+        <v>59.79</v>
       </c>
       <c r="H363">
         <f>הגדרות!B8</f>
@@ -19827,7 +19827,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>פליקס שלוקים Joyables עוף</t>
+          <t>דנטלייף לכלב מגזע קטן</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -19837,7 +19837,7 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>12620437</t>
+          <t>12606950</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
@@ -19846,10 +19846,10 @@
         </is>
       </c>
       <c r="F364" t="n">
-        <v>8.49</v>
+        <v>10.2</v>
       </c>
       <c r="G364" t="n">
-        <v>10.02</v>
+        <v>12.04</v>
       </c>
       <c r="H364">
         <f>הגדרות!B8</f>
@@ -19880,7 +19880,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>פליקס שלוקים Joyables סלמון</t>
+          <t>דנטלייף לכלב מגזע בינוני</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
@@ -19890,7 +19890,7 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>12620438</t>
+          <t>12606926</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
@@ -19899,10 +19899,10 @@
         </is>
       </c>
       <c r="F365" t="n">
-        <v>8.49</v>
+        <v>10.2</v>
       </c>
       <c r="G365" t="n">
-        <v>10.02</v>
+        <v>12.04</v>
       </c>
       <c r="H365">
         <f>הגדרות!B8</f>
@@ -19933,7 +19933,7 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>פליקס שלוקים Joyables ברווז</t>
+          <t>דנטלייף לכלב מגזע גדול</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -19943,7 +19943,7 @@
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>12620419</t>
+          <t>12606948</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
@@ -19952,10 +19952,10 @@
         </is>
       </c>
       <c r="F366" t="n">
-        <v>8.49</v>
+        <v>10.2</v>
       </c>
       <c r="G366" t="n">
-        <v>10.02</v>
+        <v>12.04</v>
       </c>
       <c r="H366">
         <f>הגדרות!B8</f>
@@ -19986,7 +19986,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>פרו פלאן חטיפי DentalCare לכלב מגזע קטן</t>
+          <t>דנטלייף חתול עוף</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -19996,7 +19996,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>12604543</t>
+          <t>12607325</t>
         </is>
       </c>
       <c r="E367" t="inlineStr">
@@ -20005,10 +20005,10 @@
         </is>
       </c>
       <c r="F367" t="n">
-        <v>25.64</v>
+        <v>6.5</v>
       </c>
       <c r="G367" t="n">
-        <v>30.26</v>
+        <v>7.67</v>
       </c>
       <c r="H367">
         <f>הגדרות!B8</f>
@@ -20039,7 +20039,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>פרו פלאן חטיפי DentalCare לכלב מגזע בינוני</t>
+          <t>דנטלייף חתול סלמון</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -20049,7 +20049,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>12604772</t>
+          <t>12607342</t>
         </is>
       </c>
       <c r="E368" t="inlineStr">
@@ -20058,10 +20058,10 @@
         </is>
       </c>
       <c r="F368" t="n">
-        <v>25.64</v>
+        <v>6.5</v>
       </c>
       <c r="G368" t="n">
-        <v>30.26</v>
+        <v>7.67</v>
       </c>
       <c r="H368">
         <f>הגדרות!B8</f>
@@ -20092,7 +20092,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>פרו פלאן חטיפי DentalCare לכלב מגזע גדול</t>
+          <t>פליקס שלוקים Joyables עוף</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -20102,7 +20102,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>12604733</t>
+          <t>12620437</t>
         </is>
       </c>
       <c r="E369" t="inlineStr">
@@ -20111,10 +20111,10 @@
         </is>
       </c>
       <c r="F369" t="n">
-        <v>25.64</v>
+        <v>8.49</v>
       </c>
       <c r="G369" t="n">
-        <v>30.26</v>
+        <v>10.02</v>
       </c>
       <c r="H369">
         <f>הגדרות!B8</f>
@@ -20145,7 +20145,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>דוגלי אקטיב בקר</t>
+          <t>פליקס שלוקים Joyables סלמון</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -20155,7 +20155,7 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>12466720</t>
+          <t>12620438</t>
         </is>
       </c>
       <c r="E370" t="inlineStr">
@@ -20164,10 +20164,10 @@
         </is>
       </c>
       <c r="F370" t="n">
-        <v>114.19</v>
+        <v>8.49</v>
       </c>
       <c r="G370" t="n">
-        <v>134.74</v>
+        <v>10.02</v>
       </c>
       <c r="H370">
         <f>הגדרות!B8</f>
@@ -20198,7 +20198,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>דוגלי גורים עוף</t>
+          <t>פליקס שלוקים Joyables ברווז</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -20208,7 +20208,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>12466622</t>
+          <t>12620419</t>
         </is>
       </c>
       <c r="E371" t="inlineStr">
@@ -20217,10 +20217,10 @@
         </is>
       </c>
       <c r="F371" t="n">
-        <v>41.46</v>
+        <v>8.49</v>
       </c>
       <c r="G371" t="n">
-        <v>48.92</v>
+        <v>10.02</v>
       </c>
       <c r="H371">
         <f>הגדרות!B8</f>
@@ -20251,7 +20251,7 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>דוגלי גזע קטן בקר</t>
+          <t>פרו פלאן חטיפי DentalCare לכלב מגזע קטן</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
@@ -20261,7 +20261,7 @@
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t>12613172</t>
+          <t>12604543</t>
         </is>
       </c>
       <c r="E372" t="inlineStr">
@@ -20270,10 +20270,10 @@
         </is>
       </c>
       <c r="F372" t="n">
-        <v>39.49</v>
+        <v>25.64</v>
       </c>
       <c r="G372" t="n">
-        <v>46.6</v>
+        <v>30.26</v>
       </c>
       <c r="H372">
         <f>הגדרות!B8</f>
@@ -20304,7 +20304,7 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>דוגלי בוגר עוף</t>
+          <t>פרו פלאן חטיפי DentalCare לכלב מגזע בינוני</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -20314,7 +20314,7 @@
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>12368765</t>
+          <t>12604772</t>
         </is>
       </c>
       <c r="E373" t="inlineStr">
@@ -20323,10 +20323,10 @@
         </is>
       </c>
       <c r="F373" t="n">
-        <v>37.61</v>
+        <v>25.64</v>
       </c>
       <c r="G373" t="n">
-        <v>44.38</v>
+        <v>30.26</v>
       </c>
       <c r="H373">
         <f>הגדרות!B8</f>
@@ -20357,7 +20357,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>דוגלי בוגר בקר</t>
+          <t>פרו פלאן חטיפי DentalCare לכלב מגזע גדול</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
@@ -20367,7 +20367,7 @@
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>12368766</t>
+          <t>12604733</t>
         </is>
       </c>
       <c r="E374" t="inlineStr">
@@ -20376,10 +20376,10 @@
         </is>
       </c>
       <c r="F374" t="n">
-        <v>37.61</v>
+        <v>25.64</v>
       </c>
       <c r="G374" t="n">
-        <v>44.38</v>
+        <v>30.26</v>
       </c>
       <c r="H374">
         <f>הגדרות!B8</f>
@@ -20410,7 +20410,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>דוגלי בוגר עוף</t>
+          <t>דוגלי אקטיב בקר</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -20420,7 +20420,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>12368676</t>
+          <t>12466720</t>
         </is>
       </c>
       <c r="E375" t="inlineStr">
@@ -20429,10 +20429,10 @@
         </is>
       </c>
       <c r="F375" t="n">
-        <v>108.76</v>
+        <v>114.19</v>
       </c>
       <c r="G375" t="n">
-        <v>128.34</v>
+        <v>134.74</v>
       </c>
       <c r="H375">
         <f>הגדרות!B8</f>
@@ -20463,7 +20463,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>דוגלי בוגר בקר</t>
+          <t>דוגלי גורים עוף</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -20473,7 +20473,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>12368675</t>
+          <t>12466622</t>
         </is>
       </c>
       <c r="E376" t="inlineStr">
@@ -20482,10 +20482,10 @@
         </is>
       </c>
       <c r="F376" t="n">
-        <v>108.76</v>
+        <v>41.46</v>
       </c>
       <c r="G376" t="n">
-        <v>128.34</v>
+        <v>48.92</v>
       </c>
       <c r="H376">
         <f>הגדרות!B8</f>
@@ -20505,6 +20505,271 @@
       </c>
       <c r="L376">
         <f>I376*(1+J376/100)+K376</f>
+        <v/>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>פורינה (חנויות)</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>דוגלי גזע קטן בקר</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>חטיפים</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>12613172</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="F377" t="n">
+        <v>39.49</v>
+      </c>
+      <c r="G377" t="n">
+        <v>46.6</v>
+      </c>
+      <c r="H377">
+        <f>הגדרות!B8</f>
+        <v/>
+      </c>
+      <c r="I377">
+        <f>F377*(1-H377/100)*1.18</f>
+        <v/>
+      </c>
+      <c r="J377">
+        <f>הגדרות!C8</f>
+        <v/>
+      </c>
+      <c r="K377">
+        <f>הגדרות!D8</f>
+        <v/>
+      </c>
+      <c r="L377">
+        <f>I377*(1+J377/100)+K377</f>
+        <v/>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>פורינה (חנויות)</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>דוגלי בוגר עוף</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>חטיפים</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>12368765</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="F378" t="n">
+        <v>37.61</v>
+      </c>
+      <c r="G378" t="n">
+        <v>44.38</v>
+      </c>
+      <c r="H378">
+        <f>הגדרות!B8</f>
+        <v/>
+      </c>
+      <c r="I378">
+        <f>F378*(1-H378/100)*1.18</f>
+        <v/>
+      </c>
+      <c r="J378">
+        <f>הגדרות!C8</f>
+        <v/>
+      </c>
+      <c r="K378">
+        <f>הגדרות!D8</f>
+        <v/>
+      </c>
+      <c r="L378">
+        <f>I378*(1+J378/100)+K378</f>
+        <v/>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>פורינה (חנויות)</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>דוגלי בוגר בקר</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>חטיפים</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>12368766</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="F379" t="n">
+        <v>37.61</v>
+      </c>
+      <c r="G379" t="n">
+        <v>44.38</v>
+      </c>
+      <c r="H379">
+        <f>הגדרות!B8</f>
+        <v/>
+      </c>
+      <c r="I379">
+        <f>F379*(1-H379/100)*1.18</f>
+        <v/>
+      </c>
+      <c r="J379">
+        <f>הגדרות!C8</f>
+        <v/>
+      </c>
+      <c r="K379">
+        <f>הגדרות!D8</f>
+        <v/>
+      </c>
+      <c r="L379">
+        <f>I379*(1+J379/100)+K379</f>
+        <v/>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>פורינה (חנויות)</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>דוגלי בוגר עוף</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>חטיפים</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>12368676</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="F380" t="n">
+        <v>108.76</v>
+      </c>
+      <c r="G380" t="n">
+        <v>128.34</v>
+      </c>
+      <c r="H380">
+        <f>הגדרות!B8</f>
+        <v/>
+      </c>
+      <c r="I380">
+        <f>F380*(1-H380/100)*1.18</f>
+        <v/>
+      </c>
+      <c r="J380">
+        <f>הגדרות!C8</f>
+        <v/>
+      </c>
+      <c r="K380">
+        <f>הגדרות!D8</f>
+        <v/>
+      </c>
+      <c r="L380">
+        <f>I380*(1+J380/100)+K380</f>
+        <v/>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>פורינה (חנויות)</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>דוגלי בוגר בקר</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>חטיפים</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>12368675</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="F381" t="n">
+        <v>108.76</v>
+      </c>
+      <c r="G381" t="n">
+        <v>128.34</v>
+      </c>
+      <c r="H381">
+        <f>הגדרות!B8</f>
+        <v/>
+      </c>
+      <c r="I381">
+        <f>F381*(1-H381/100)*1.18</f>
+        <v/>
+      </c>
+      <c r="J381">
+        <f>הגדרות!C8</f>
+        <v/>
+      </c>
+      <c r="K381">
+        <f>הגדרות!D8</f>
+        <v/>
+      </c>
+      <c r="L381">
+        <f>I381*(1+J381/100)+K381</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
data(vetmarket): 4 consolidated invoice PDFs (01-05/2026) -> 232 to 294 SKUs
Vetmarket publishes no price list, so its rows come from invoices. Added a
parser for the consolidated tax-invoice PDFs that takes ONLY the product name
and "מחיר ליחידה" (the list price before discount); quantity, discount and line
totals are read to locate the columns and never written out. The PDFs are not
copied to sources/ - they carry the clinic's own purchase data.

Merge across the three invoice stores now keeps the longest name per SKU
(the PDF truncates the description column) while the newest month sets price.

Data fetches revalidate (cache: no-cache) so a rebuilt list is not served stale.

Total 5763 -> 5828 items, 29 price lists.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XoJGvA8cApVXFb92aBk3Fg
</commit_message>
<xml_diff>
--- a/downloads/shop.xlsx
+++ b/downloads/shop.xlsx
@@ -579,7 +579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L381"/>
+  <dimension ref="A1:L384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -16801,37 +16801,37 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>מדי-מרקט</t>
+          <t>וטמרקט</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>@ סדיניה 35 60X90 יח' TENA BED @</t>
+          <t>חול Kit4Cat</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>אביזרים</t>
+          <t>חול ושירותים</t>
         </is>
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>33262-1</t>
+          <t>460001</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="F307" t="n">
-        <v>31.36</v>
+        <v>40</v>
       </c>
       <c r="G307" t="n">
-        <v>37</v>
+        <v>47.2</v>
       </c>
       <c r="H307">
-        <f>הגדרות!B6</f>
+        <f>הגדרות!B5</f>
         <v/>
       </c>
       <c r="I307">
@@ -16839,11 +16839,11 @@
         <v/>
       </c>
       <c r="J307">
-        <f>הגדרות!C6</f>
+        <f>הגדרות!C5</f>
         <v/>
       </c>
       <c r="K307">
-        <f>הגדרות!D6</f>
+        <f>הגדרות!D5</f>
         <v/>
       </c>
       <c r="L307">
@@ -16854,37 +16854,37 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>מדי-מרקט</t>
+          <t>וטמרקט</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>ANTIGONE WIPES 19*20 500</t>
+          <t>חטיף ווג'ידנט 15 Small יחידות, 228 גרם</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>חטיפים</t>
         </is>
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>M0002020</t>
+          <t>47307869</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="F308" t="n">
-        <v>71.42</v>
+        <v>19</v>
       </c>
       <c r="G308" t="n">
-        <v>84.27</v>
+        <v>22.42</v>
       </c>
       <c r="H308">
-        <f>הגדרות!B6</f>
+        <f>הגדרות!B5</f>
         <v/>
       </c>
       <c r="I308">
@@ -16892,11 +16892,11 @@
         <v/>
       </c>
       <c r="J308">
-        <f>הגדרות!C6</f>
+        <f>הגדרות!C5</f>
         <v/>
       </c>
       <c r="K308">
-        <f>הגדרות!D6</f>
+        <f>הגדרות!D5</f>
         <v/>
       </c>
       <c r="L308">
@@ -16907,37 +16907,37 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>מדי-מרקט</t>
+          <t>וטמרקט</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>ANTIGONE WIPES 20*20 200</t>
+          <t>חטיף ווג'ידנט 15 Large יחידות, 502 גרם</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>חטיפים</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>100003</t>
+          <t>47307871</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="F309" t="n">
-        <v>30.32</v>
+        <v>30</v>
       </c>
       <c r="G309" t="n">
-        <v>35.78</v>
+        <v>35.4</v>
       </c>
       <c r="H309">
-        <f>הגדרות!B6</f>
+        <f>הגדרות!B5</f>
         <v/>
       </c>
       <c r="I309">
@@ -16945,11 +16945,11 @@
         <v/>
       </c>
       <c r="J309">
-        <f>הגדרות!C6</f>
+        <f>הגדרות!C5</f>
         <v/>
       </c>
       <c r="K309">
-        <f>הגדרות!D6</f>
+        <f>הגדרות!D5</f>
         <v/>
       </c>
       <c r="L309">
@@ -16965,17 +16965,17 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>CETRIN 1 LITTER SOL</t>
+          <t>@ סדיניה 35 60X90 יח' TENA BED @</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>חול ושירותים</t>
+          <t>אביזרים</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>33365</t>
+          <t>33262-1</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
@@ -16984,10 +16984,10 @@
         </is>
       </c>
       <c r="F310" t="n">
-        <v>30.84</v>
+        <v>31.36</v>
       </c>
       <c r="G310" t="n">
-        <v>36.39</v>
+        <v>37</v>
       </c>
       <c r="H310">
         <f>הגדרות!B6</f>
@@ -17018,7 +17018,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>DOUXO S3 CALM MOUSSE 150 ML</t>
+          <t>ANTIGONE WIPES 19*20 500</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -17028,7 +17028,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>81-105</t>
+          <t>M0002020</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
@@ -17037,10 +17037,10 @@
         </is>
       </c>
       <c r="F311" t="n">
-        <v>58.47</v>
+        <v>71.42</v>
       </c>
       <c r="G311" t="n">
-        <v>69</v>
+        <v>84.27</v>
       </c>
       <c r="H311">
         <f>הגדרות!B6</f>
@@ -17071,7 +17071,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>DOUXO S3 PYO MOUSSE 150 ML</t>
+          <t>ANTIGONE WIPES 20*20 200</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -17081,7 +17081,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>81-101</t>
+          <t>100003</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
@@ -17090,10 +17090,10 @@
         </is>
       </c>
       <c r="F312" t="n">
-        <v>58.47</v>
+        <v>30.32</v>
       </c>
       <c r="G312" t="n">
-        <v>69</v>
+        <v>35.78</v>
       </c>
       <c r="H312">
         <f>הגדרות!B6</f>
@@ -17124,17 +17124,17 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>DOUXO S3 PYO PADS</t>
+          <t>CETRIN 1 LITTER SOL</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>חול ושירותים</t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>81-107</t>
+          <t>33365</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
@@ -17143,10 +17143,10 @@
         </is>
       </c>
       <c r="F313" t="n">
-        <v>36.44</v>
+        <v>30.84</v>
       </c>
       <c r="G313" t="n">
-        <v>43</v>
+        <v>36.39</v>
       </c>
       <c r="H313">
         <f>הגדרות!B6</f>
@@ -17177,7 +17177,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>DOUXO S3 SEB MOUSSE 150 ML</t>
+          <t>DOUXO S3 CALM MOUSSE 150 ML</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -17187,7 +17187,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>81-103</t>
+          <t>81-105</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
@@ -17230,17 +17230,17 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Easy Go 500 Litter - איזי גו</t>
+          <t>DOUXO S3 PYO MOUSSE 150 ML</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>חול ושירותים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>18033-1</t>
+          <t>81-101</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
@@ -17249,10 +17249,10 @@
         </is>
       </c>
       <c r="F315" t="n">
-        <v>14.32</v>
+        <v>58.47</v>
       </c>
       <c r="G315" t="n">
-        <v>16.9</v>
+        <v>69</v>
       </c>
       <c r="H315">
         <f>הגדרות!B6</f>
@@ -17283,17 +17283,17 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Pinchers 45chews peanut butter pill hiding treat</t>
+          <t>DOUXO S3 PYO PADS</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>חטיפים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>090062J.045</t>
+          <t>81-107</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
@@ -17302,10 +17302,10 @@
         </is>
       </c>
       <c r="F316" t="n">
-        <v>22.3</v>
+        <v>36.44</v>
       </c>
       <c r="G316" t="n">
-        <v>26.31</v>
+        <v>43</v>
       </c>
       <c r="H316">
         <f>הגדרות!B6</f>
@@ -17336,17 +17336,17 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>אלונקה רכה מתקפלת NAR QuikLitter</t>
+          <t>DOUXO S3 SEB MOUSSE 150 ML</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>חול ושירותים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>4105</t>
+          <t>81-103</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
@@ -17355,10 +17355,10 @@
         </is>
       </c>
       <c r="F317" t="n">
-        <v>194.49</v>
+        <v>58.47</v>
       </c>
       <c r="G317" t="n">
-        <v>229.5</v>
+        <v>69</v>
       </c>
       <c r="H317">
         <f>הגדרות!B6</f>
@@ -17389,17 +17389,17 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>כלוב נשיאה אטלס 10 ללא מזרון Ferplast</t>
+          <t>Easy Go 500 Litter - איזי גו</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>חול ושירותים</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>5550279</t>
+          <t>18033-1</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
@@ -17408,10 +17408,10 @@
         </is>
       </c>
       <c r="F318" t="n">
-        <v>50.85</v>
+        <v>14.32</v>
       </c>
       <c r="G318" t="n">
-        <v>60</v>
+        <v>16.9</v>
       </c>
       <c r="H318">
         <f>הגדרות!B6</f>
@@ -17442,17 +17442,17 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>כלוב נשיאה אטלס 20 ללא מזרון Ferplast</t>
+          <t>Pinchers 45chews peanut butter pill hiding treat</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>חטיפים</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>5550280</t>
+          <t>090062J.045</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
@@ -17461,10 +17461,10 @@
         </is>
       </c>
       <c r="F319" t="n">
-        <v>88.14</v>
+        <v>22.3</v>
       </c>
       <c r="G319" t="n">
-        <v>104</v>
+        <v>26.31</v>
       </c>
       <c r="H319">
         <f>הגדרות!B6</f>
@@ -17495,17 +17495,17 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>מברשת רחצת ידיים לפני ניתוח, סטר', מדיקפרו</t>
+          <t>אלונקה רכה מתקפלת NAR QuikLitter</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>חול ושירותים</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>3694</t>
+          <t>4105</t>
         </is>
       </c>
       <c r="E320" t="inlineStr">
@@ -17514,10 +17514,10 @@
         </is>
       </c>
       <c r="F320" t="n">
-        <v>0.87</v>
+        <v>194.49</v>
       </c>
       <c r="G320" t="n">
-        <v>1.03</v>
+        <v>229.5</v>
       </c>
       <c r="H320">
         <f>הגדרות!B6</f>
@@ -17548,7 +17548,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>מגבונים - Clinell sporicidal wipesn 1/6</t>
+          <t>כלוב נשיאה אטלס 10 ללא מזרון Ferplast</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -17558,7 +17558,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>CS25</t>
+          <t>5550279</t>
         </is>
       </c>
       <c r="E321" t="inlineStr">
@@ -17567,10 +17567,10 @@
         </is>
       </c>
       <c r="F321" t="n">
-        <v>156.78</v>
+        <v>50.85</v>
       </c>
       <c r="G321" t="n">
-        <v>185</v>
+        <v>60</v>
       </c>
       <c r="H321">
         <f>הגדרות!B6</f>
@@ -17601,7 +17601,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>מגבונים - Clinell Universal wipes clip pack 50</t>
+          <t>כלוב נשיאה אטלס 20 ללא מזרון Ferplast</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -17611,7 +17611,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>11050</t>
+          <t>5550280</t>
         </is>
       </c>
       <c r="E322" t="inlineStr">
@@ -17620,10 +17620,10 @@
         </is>
       </c>
       <c r="F322" t="n">
-        <v>9.25</v>
+        <v>88.14</v>
       </c>
       <c r="G322" t="n">
-        <v>10.92</v>
+        <v>104</v>
       </c>
       <c r="H322">
         <f>הגדרות!B6</f>
@@ -17654,7 +17654,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>מגבונים - Clinell Universal Wipes pack of 200</t>
+          <t>מברשת רחצת ידיים לפני ניתוח, סטר', מדיקפרו</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -17664,7 +17664,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>11200</t>
+          <t>3694</t>
         </is>
       </c>
       <c r="E323" t="inlineStr">
@@ -17673,10 +17673,10 @@
         </is>
       </c>
       <c r="F323" t="n">
-        <v>19.92</v>
+        <v>0.87</v>
       </c>
       <c r="G323" t="n">
-        <v>23.5</v>
+        <v>1.03</v>
       </c>
       <c r="H323">
         <f>הגדרות!B6</f>
@@ -17707,7 +17707,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>מגבונים מדי-קלין אקסטרה עבים מועשר באלוורה 500 יח 20X16 ס"מ</t>
+          <t>מגבונים - Clinell sporicidal wipesn 1/6</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -17717,7 +17717,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>128697</t>
+          <t>CS25</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
@@ -17726,10 +17726,10 @@
         </is>
       </c>
       <c r="F324" t="n">
-        <v>22.88</v>
+        <v>156.78</v>
       </c>
       <c r="G324" t="n">
-        <v>27</v>
+        <v>185</v>
       </c>
       <c r="H324">
         <f>הגדרות!B6</f>
@@ -17760,7 +17760,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>מגבונים מדי-קלין מועשרים באלוורה 500 יח' 28X20 ס"מ</t>
+          <t>מגבונים - Clinell Universal wipes clip pack 50</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -17770,7 +17770,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>128695</t>
+          <t>11050</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
@@ -17779,10 +17779,10 @@
         </is>
       </c>
       <c r="F325" t="n">
-        <v>22.88</v>
+        <v>9.25</v>
       </c>
       <c r="G325" t="n">
-        <v>27</v>
+        <v>10.92</v>
       </c>
       <c r="H325">
         <f>הגדרות!B6</f>
@@ -17813,17 +17813,17 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>מיטה חשמלית דגם GUESS 402 מעקה מגלוון</t>
+          <t>מגבונים - Clinell Universal Wipes pack of 200</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>אביזרים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>883135</t>
+          <t>11200</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
@@ -17832,10 +17832,10 @@
         </is>
       </c>
       <c r="F326" t="n">
-        <v>6288.14</v>
+        <v>19.92</v>
       </c>
       <c r="G326" t="n">
-        <v>7420</v>
+        <v>23.5</v>
       </c>
       <c r="H326">
         <f>הגדרות!B6</f>
@@ -17866,7 +17866,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>מספריים אל חלד לציפורניים REISZ</t>
+          <t>מגבונים מדי-קלין אקסטרה עבים מועשר באלוורה 500 יח 20X16 ס"מ</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -17876,7 +17876,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>434457</t>
+          <t>128697</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
@@ -17885,10 +17885,10 @@
         </is>
       </c>
       <c r="F327" t="n">
-        <v>21.17</v>
+        <v>22.88</v>
       </c>
       <c r="G327" t="n">
-        <v>24.98</v>
+        <v>27</v>
       </c>
       <c r="H327">
         <f>הגדרות!B6</f>
@@ -17919,7 +17919,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>משושת ג'ל 500 מ"ל פוליגונום רב תכליתי Herbaderm</t>
+          <t>מגבונים מדי-קלין מועשרים באלוורה 500 יח' 28X20 ס"מ</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -17929,7 +17929,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>67-105</t>
+          <t>128695</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
@@ -17938,10 +17938,10 @@
         </is>
       </c>
       <c r="F328" t="n">
-        <v>157.63</v>
+        <v>22.88</v>
       </c>
       <c r="G328" t="n">
-        <v>186</v>
+        <v>27</v>
       </c>
       <c r="H328">
         <f>הגדרות!B6</f>
@@ -17972,17 +17972,17 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>משושת קרם 500 מ"ל פוליגונום רב תכליתי Herbaderm</t>
+          <t>מיטה חשמלית דגם GUESS 402 מעקה מגלוון</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>אביזרים</t>
         </is>
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>67-103</t>
+          <t>883135</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
@@ -17991,10 +17991,10 @@
         </is>
       </c>
       <c r="F329" t="n">
-        <v>157.63</v>
+        <v>6288.14</v>
       </c>
       <c r="G329" t="n">
-        <v>186</v>
+        <v>7420</v>
       </c>
       <c r="H329">
         <f>הגדרות!B6</f>
@@ -18025,7 +18025,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>נייר לניגוב עדשות מיקרוסקופ 1159 1/280 Kimwipes</t>
+          <t>מספריים אל חלד לציפורניים REISZ</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -18035,7 +18035,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>3422</t>
+          <t>434457</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
@@ -18044,10 +18044,10 @@
         </is>
       </c>
       <c r="F330" t="n">
-        <v>26.44</v>
+        <v>21.17</v>
       </c>
       <c r="G330" t="n">
-        <v>31.2</v>
+        <v>24.98</v>
       </c>
       <c r="H330">
         <f>הגדרות!B6</f>
@@ -18078,17 +18078,17 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>סיר לילה פלסטיק/ מיטה גדול עם ידית, מדיקפרו</t>
+          <t>משושת ג'ל 500 מ"ל פוליגונום רב תכליתי Herbaderm</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>אביזרים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>4055</t>
+          <t>67-105</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
@@ -18097,10 +18097,10 @@
         </is>
       </c>
       <c r="F331" t="n">
-        <v>11.86</v>
+        <v>157.63</v>
       </c>
       <c r="G331" t="n">
-        <v>14</v>
+        <v>186</v>
       </c>
       <c r="H331">
         <f>הגדרות!B6</f>
@@ -18131,7 +18131,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>קוצץ ציפורניים, מדיקפרו</t>
+          <t>משושת קרם 500 מ"ל פוליגונום רב תכליתי Herbaderm</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -18141,7 +18141,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>17709</t>
+          <t>67-103</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
@@ -18150,10 +18150,10 @@
         </is>
       </c>
       <c r="F332" t="n">
-        <v>3.32</v>
+        <v>157.63</v>
       </c>
       <c r="G332" t="n">
-        <v>3.92</v>
+        <v>186</v>
       </c>
       <c r="H332">
         <f>הגדרות!B6</f>
@@ -18184,7 +18184,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>ראש למכונת תספורת (סכין) 40 - 0.25 מ"מ LAUBE</t>
+          <t>נייר לניגוב עדשות מיקרוסקופ 1159 1/280 Kimwipes</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -18194,7 +18194,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>80662</t>
+          <t>3422</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
@@ -18203,10 +18203,10 @@
         </is>
       </c>
       <c r="F333" t="n">
-        <v>120.13</v>
+        <v>26.44</v>
       </c>
       <c r="G333" t="n">
-        <v>141.75</v>
+        <v>31.2</v>
       </c>
       <c r="H333">
         <f>הגדרות!B6</f>
@@ -18237,7 +18237,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>רצועה ללוח גב צבע כתום עם אבזם מתכת</t>
+          <t>סיר לילה פלסטיק/ מיטה גדול עם ידית, מדיקפרו</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -18247,7 +18247,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>16155</t>
+          <t>4055</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -18256,10 +18256,10 @@
         </is>
       </c>
       <c r="F334" t="n">
-        <v>71.19</v>
+        <v>11.86</v>
       </c>
       <c r="G334" t="n">
-        <v>84</v>
+        <v>14</v>
       </c>
       <c r="H334">
         <f>הגדרות!B6</f>
@@ -18290,17 +18290,17 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>רצועה לתמיכה למסכת טרכוסטומי L</t>
+          <t>קוצץ ציפורניים, מדיקפרו</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>אביזרים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>7985</t>
+          <t>17709</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
@@ -18309,10 +18309,10 @@
         </is>
       </c>
       <c r="F335" t="n">
-        <v>5.91</v>
+        <v>3.32</v>
       </c>
       <c r="G335" t="n">
-        <v>6.97</v>
+        <v>3.92</v>
       </c>
       <c r="H335">
         <f>הגדרות!B6</f>
@@ -18343,17 +18343,17 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>רצועה לתמיכה למסכת טרכוסטומי M</t>
+          <t>ראש למכונת תספורת (סכין) 40 - 0.25 מ"מ LAUBE</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>אביזרים</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>7987</t>
+          <t>80662</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
@@ -18362,10 +18362,10 @@
         </is>
       </c>
       <c r="F336" t="n">
-        <v>6.19</v>
+        <v>120.13</v>
       </c>
       <c r="G336" t="n">
-        <v>7.3</v>
+        <v>141.75</v>
       </c>
       <c r="H336">
         <f>הגדרות!B6</f>
@@ -18396,7 +18396,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>רצועה לתמיכה למסכת טרכוסטומי XL</t>
+          <t>רצועה ללוח גב צבע כתום עם אבזם מתכת</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -18406,7 +18406,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>7986</t>
+          <t>16155</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
@@ -18415,10 +18415,10 @@
         </is>
       </c>
       <c r="F337" t="n">
-        <v>6.36</v>
+        <v>71.19</v>
       </c>
       <c r="G337" t="n">
-        <v>7.5</v>
+        <v>84</v>
       </c>
       <c r="H337">
         <f>הגדרות!B6</f>
@@ -18444,37 +18444,37 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>פט-וט ביומד</t>
+          <t>מדי-מרקט</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Keto Tris Finger Wipes 50 units</t>
+          <t>רצועה לתמיכה למסכת טרכוסטומי L</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>אביזרים</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>DERMA-SP1330</t>
+          <t>7985</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F338" t="n">
-        <v>59</v>
+        <v>5.91</v>
       </c>
       <c r="G338" t="n">
-        <v>69.62</v>
+        <v>6.97</v>
       </c>
       <c r="H338">
-        <f>הגדרות!B7</f>
+        <f>הגדרות!B6</f>
         <v/>
       </c>
       <c r="I338">
@@ -18482,11 +18482,11 @@
         <v/>
       </c>
       <c r="J338">
-        <f>הגדרות!C7</f>
+        <f>הגדרות!C6</f>
         <v/>
       </c>
       <c r="K338">
-        <f>הגדרות!D7</f>
+        <f>הגדרות!D6</f>
         <v/>
       </c>
       <c r="L338">
@@ -18497,37 +18497,37 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>פט-וט ביומד</t>
+          <t>מדי-מרקט</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Tris Ophto Wipes 50ct</t>
+          <t>רצועה לתמיכה למסכת טרכוסטומי M</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>טיפוח והיגיינה</t>
+          <t>אביזרים</t>
         </is>
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>DZOO-TWX</t>
+          <t>7987</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F339" t="n">
-        <v>58</v>
+        <v>6.19</v>
       </c>
       <c r="G339" t="n">
-        <v>68.44</v>
+        <v>7.3</v>
       </c>
       <c r="H339">
-        <f>הגדרות!B7</f>
+        <f>הגדרות!B6</f>
         <v/>
       </c>
       <c r="I339">
@@ -18535,11 +18535,11 @@
         <v/>
       </c>
       <c r="J339">
-        <f>הגדרות!C7</f>
+        <f>הגדרות!C6</f>
         <v/>
       </c>
       <c r="K339">
-        <f>הגדרות!D7</f>
+        <f>הגדרות!D6</f>
         <v/>
       </c>
       <c r="L339">
@@ -18550,37 +18550,37 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>פט-וט ביומד</t>
+          <t>מדי-מרקט</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Pill Splitter</t>
+          <t>רצועה לתמיכה למסכת טרכוסטומי XL</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>חול ושירותים</t>
+          <t>אביזרים</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>FIONA-821070-1</t>
+          <t>7986</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="F340" t="n">
-        <v>7</v>
+        <v>6.36</v>
       </c>
       <c r="G340" t="n">
-        <v>8.26</v>
+        <v>7.5</v>
       </c>
       <c r="H340">
-        <f>הגדרות!B7</f>
+        <f>הגדרות!B6</f>
         <v/>
       </c>
       <c r="I340">
@@ -18588,11 +18588,11 @@
         <v/>
       </c>
       <c r="J340">
-        <f>הגדרות!C7</f>
+        <f>הגדרות!C6</f>
         <v/>
       </c>
       <c r="K340">
-        <f>הגדרות!D7</f>
+        <f>הגדרות!D6</f>
         <v/>
       </c>
       <c r="L340">
@@ -18608,17 +18608,17 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Calming Spray 200ml</t>
+          <t>Keto Tris Finger Wipes 50 units</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>הרגעה</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>PR-79583</t>
+          <t>DERMA-SP1330</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
@@ -18627,10 +18627,10 @@
         </is>
       </c>
       <c r="F341" t="n">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="G341" t="n">
-        <v>54.28</v>
+        <v>69.62</v>
       </c>
       <c r="H341">
         <f>הגדרות!B7</f>
@@ -18661,17 +18661,17 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Mini Calming Spray 15ml</t>
+          <t>Tris Ophto Wipes 50ct</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>הרגעה</t>
+          <t>טיפוח והיגיינה</t>
         </is>
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>PR-79664</t>
+          <t>DZOO-TWX</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
@@ -18680,10 +18680,10 @@
         </is>
       </c>
       <c r="F342" t="n">
-        <v>18</v>
+        <v>58</v>
       </c>
       <c r="G342" t="n">
-        <v>21.24</v>
+        <v>68.44</v>
       </c>
       <c r="H342">
         <f>הגדרות!B7</f>
@@ -18714,17 +18714,17 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Battery Atomizer Refill 300ml</t>
+          <t>Pill Splitter</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>הרגעה</t>
+          <t>חול ושירותים</t>
         </is>
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>PR-79744</t>
+          <t>FIONA-821070-1</t>
         </is>
       </c>
       <c r="E343" t="inlineStr">
@@ -18733,10 +18733,10 @@
         </is>
       </c>
       <c r="F343" t="n">
-        <v>56</v>
+        <v>7</v>
       </c>
       <c r="G343" t="n">
-        <v>66.08</v>
+        <v>8.26</v>
       </c>
       <c r="H343">
         <f>הגדרות!B7</f>
@@ -18767,7 +18767,7 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Battery Atomizer</t>
+          <t>Calming Spray 200ml</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
@@ -18777,7 +18777,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>PR-79745</t>
+          <t>PR-79583</t>
         </is>
       </c>
       <c r="E344" t="inlineStr">
@@ -18786,10 +18786,10 @@
         </is>
       </c>
       <c r="F344" t="n">
-        <v>185</v>
+        <v>46</v>
       </c>
       <c r="G344" t="n">
-        <v>218.3</v>
+        <v>54.28</v>
       </c>
       <c r="H344">
         <f>הגדרות!B7</f>
@@ -18820,7 +18820,7 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Calming Wipe Sachet (12)</t>
+          <t>Mini Calming Spray 15ml</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -18830,7 +18830,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>PR-79881</t>
+          <t>PR-79664</t>
         </is>
       </c>
       <c r="E345" t="inlineStr">
@@ -18873,17 +18873,17 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Boredom Buster forager kit</t>
+          <t>Battery Atomizer Refill 300ml</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>צעצועים</t>
+          <t>הרגעה</t>
         </is>
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>PR-80128</t>
+          <t>PR-79744</t>
         </is>
       </c>
       <c r="E346" t="inlineStr">
@@ -18892,10 +18892,10 @@
         </is>
       </c>
       <c r="F346" t="n">
-        <v>105</v>
+        <v>56</v>
       </c>
       <c r="G346" t="n">
-        <v>123.9</v>
+        <v>66.08</v>
       </c>
       <c r="H346">
         <f>הגדרות!B7</f>
@@ -18926,7 +18926,7 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Calming Bandana Kit EXTRA SMALL</t>
+          <t>Battery Atomizer</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -18936,7 +18936,7 @@
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>PR-79959</t>
+          <t>PR-79745</t>
         </is>
       </c>
       <c r="E347" t="inlineStr">
@@ -18945,10 +18945,10 @@
         </is>
       </c>
       <c r="F347" t="n">
-        <v>44</v>
+        <v>185</v>
       </c>
       <c r="G347" t="n">
-        <v>51.92</v>
+        <v>218.3</v>
       </c>
       <c r="H347">
         <f>הגדרות!B7</f>
@@ -18979,7 +18979,7 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Calming Bandana Kit SMALL</t>
+          <t>Calming Wipe Sachet (12)</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -18989,7 +18989,7 @@
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>PR-79960</t>
+          <t>PR-79881</t>
         </is>
       </c>
       <c r="E348" t="inlineStr">
@@ -18998,10 +18998,10 @@
         </is>
       </c>
       <c r="F348" t="n">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="G348" t="n">
-        <v>51.92</v>
+        <v>21.24</v>
       </c>
       <c r="H348">
         <f>הגדרות!B7</f>
@@ -19032,17 +19032,17 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Calming Bandana Kit MEDIUM</t>
+          <t>Boredom Buster forager kit</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>הרגעה</t>
+          <t>צעצועים</t>
         </is>
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>PR-79961</t>
+          <t>PR-80128</t>
         </is>
       </c>
       <c r="E349" t="inlineStr">
@@ -19051,10 +19051,10 @@
         </is>
       </c>
       <c r="F349" t="n">
-        <v>44</v>
+        <v>105</v>
       </c>
       <c r="G349" t="n">
-        <v>51.92</v>
+        <v>123.9</v>
       </c>
       <c r="H349">
         <f>הגדרות!B7</f>
@@ -19085,7 +19085,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Calming Bandana Kit LARGE</t>
+          <t>Calming Bandana Kit EXTRA SMALL</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -19095,7 +19095,7 @@
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>PR-79962</t>
+          <t>PR-79959</t>
         </is>
       </c>
       <c r="E350" t="inlineStr">
@@ -19138,7 +19138,7 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Calming Spray 400ml – PROF. PACK</t>
+          <t>Calming Bandana Kit SMALL</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -19148,7 +19148,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>PR-79983</t>
+          <t>PR-79960</t>
         </is>
       </c>
       <c r="E351" t="inlineStr">
@@ -19157,10 +19157,10 @@
         </is>
       </c>
       <c r="F351" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="G351" t="n">
-        <v>71.98</v>
+        <v>51.92</v>
       </c>
       <c r="H351">
         <f>הגדרות!B7</f>
@@ -19186,37 +19186,37 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>פורינה (חנויות)</t>
+          <t>פט-וט ביומד</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס אוריגי'נל קראנץ</t>
+          <t>Calming Bandana Kit MEDIUM</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>חטיפים</t>
+          <t>הרגעה</t>
         </is>
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>12348261</t>
+          <t>PR-79961</t>
         </is>
       </c>
       <c r="E352" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="F352" t="n">
-        <v>8.18</v>
+        <v>44</v>
       </c>
       <c r="G352" t="n">
-        <v>9.65</v>
+        <v>51.92</v>
       </c>
       <c r="H352">
-        <f>הגדרות!B8</f>
+        <f>הגדרות!B7</f>
         <v/>
       </c>
       <c r="I352">
@@ -19224,11 +19224,11 @@
         <v/>
       </c>
       <c r="J352">
-        <f>הגדרות!C8</f>
+        <f>הגדרות!C7</f>
         <v/>
       </c>
       <c r="K352">
-        <f>הגדרות!D8</f>
+        <f>הגדרות!D7</f>
         <v/>
       </c>
       <c r="L352">
@@ -19239,37 +19239,37 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>פורינה (חנויות)</t>
+          <t>פט-וט ביומד</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס מיקס גריל קראנץ</t>
+          <t>Calming Bandana Kit LARGE</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>חטיפים</t>
+          <t>הרגעה</t>
         </is>
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>12348037</t>
+          <t>PR-79962</t>
         </is>
       </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="F353" t="n">
-        <v>8.18</v>
+        <v>44</v>
       </c>
       <c r="G353" t="n">
-        <v>9.65</v>
+        <v>51.92</v>
       </c>
       <c r="H353">
-        <f>הגדרות!B8</f>
+        <f>הגדרות!B7</f>
         <v/>
       </c>
       <c r="I353">
@@ -19277,11 +19277,11 @@
         <v/>
       </c>
       <c r="J353">
-        <f>הגדרות!C8</f>
+        <f>הגדרות!C7</f>
         <v/>
       </c>
       <c r="K353">
-        <f>הגדרות!D8</f>
+        <f>הגדרות!D7</f>
         <v/>
       </c>
       <c r="L353">
@@ -19292,37 +19292,37 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>פורינה (חנויות)</t>
+          <t>פט-וט ביומד</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס מעדני ים קראנץ</t>
+          <t>Calming Spray 400ml – PROF. PACK</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>חטיפים</t>
+          <t>הרגעה</t>
         </is>
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>12364507</t>
+          <t>PR-79983</t>
         </is>
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="F354" t="n">
-        <v>8.18</v>
+        <v>61</v>
       </c>
       <c r="G354" t="n">
-        <v>9.65</v>
+        <v>71.98</v>
       </c>
       <c r="H354">
-        <f>הגדרות!B8</f>
+        <f>הגדרות!B7</f>
         <v/>
       </c>
       <c r="I354">
@@ -19330,11 +19330,11 @@
         <v/>
       </c>
       <c r="J354">
-        <f>הגדרות!C8</f>
+        <f>הגדרות!C7</f>
         <v/>
       </c>
       <c r="K354">
-        <f>הגדרות!D8</f>
+        <f>הגדרות!D7</f>
         <v/>
       </c>
       <c r="L354">
@@ -19350,7 +19350,7 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס פיקניק קרנץ</t>
+          <t>פריסקיז פארטי מיקס אוריגי'נל קראנץ</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -19360,7 +19360,7 @@
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>12368621</t>
+          <t>12348261</t>
         </is>
       </c>
       <c r="E355" t="inlineStr">
@@ -19403,7 +19403,7 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס קרייזי צ'יז</t>
+          <t>פריסקיז פארטי מיקס מיקס גריל קראנץ</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -19413,7 +19413,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>12528489</t>
+          <t>12348037</t>
         </is>
       </c>
       <c r="E356" t="inlineStr">
@@ -19456,7 +19456,7 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס מאנץ' בוקר</t>
+          <t>פריסקיז פארטי מיקס מעדני ים קראנץ</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -19466,7 +19466,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>12280472</t>
+          <t>12364507</t>
         </is>
       </c>
       <c r="E357" t="inlineStr">
@@ -19509,7 +19509,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס הודו</t>
+          <t>פריסקיז פארטי מיקס פיקניק קרנץ</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -19519,7 +19519,7 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>12332654</t>
+          <t>12368621</t>
         </is>
       </c>
       <c r="E358" t="inlineStr">
@@ -19562,7 +19562,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>פריסקיז פארטי מיקס עוף</t>
+          <t>פריסקיז פארטי מיקס קרייזי צ'יז</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -19572,7 +19572,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>12332617</t>
+          <t>12528489</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
@@ -19615,7 +19615,7 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>פריסקיז פלייפולס סלמון ושרימפס</t>
+          <t>פריסקיז פארטי מיקס מאנץ' בוקר</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -19625,7 +19625,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>12534203</t>
+          <t>12280472</t>
         </is>
       </c>
       <c r="E360" t="inlineStr">
@@ -19668,7 +19668,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>פריסקיז פלייפולס עוף וכבד</t>
+          <t>פריסקיז פארטי מיקס הודו</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -19678,7 +19678,7 @@
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>12534194</t>
+          <t>12332654</t>
         </is>
       </c>
       <c r="E361" t="inlineStr">
@@ -19721,7 +19721,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>פריסקיז צנצנת פארטי מיקס מעדני ים קראנץ</t>
+          <t>פריסקיז פארטי מיקס עוף</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -19731,7 +19731,7 @@
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>12364794</t>
+          <t>12332617</t>
         </is>
       </c>
       <c r="E362" t="inlineStr">
@@ -19740,10 +19740,10 @@
         </is>
       </c>
       <c r="F362" t="n">
-        <v>50.67</v>
+        <v>8.18</v>
       </c>
       <c r="G362" t="n">
-        <v>59.79</v>
+        <v>9.65</v>
       </c>
       <c r="H362">
         <f>הגדרות!B8</f>
@@ -19774,7 +19774,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>פריסקיז צנצנת פארטי מיקס אוריגי'נל קראנץ</t>
+          <t>פריסקיז פלייפולס סלמון ושרימפס</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -19784,7 +19784,7 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>12349730</t>
+          <t>12534203</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
@@ -19793,10 +19793,10 @@
         </is>
       </c>
       <c r="F363" t="n">
-        <v>50.67</v>
+        <v>8.18</v>
       </c>
       <c r="G363" t="n">
-        <v>59.79</v>
+        <v>9.65</v>
       </c>
       <c r="H363">
         <f>הגדרות!B8</f>
@@ -19827,7 +19827,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>דנטלייף לכלב מגזע קטן</t>
+          <t>פריסקיז פלייפולס עוף וכבד</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -19837,7 +19837,7 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>12606950</t>
+          <t>12534194</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
@@ -19846,10 +19846,10 @@
         </is>
       </c>
       <c r="F364" t="n">
-        <v>10.2</v>
+        <v>8.18</v>
       </c>
       <c r="G364" t="n">
-        <v>12.04</v>
+        <v>9.65</v>
       </c>
       <c r="H364">
         <f>הגדרות!B8</f>
@@ -19880,7 +19880,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>דנטלייף לכלב מגזע בינוני</t>
+          <t>פריסקיז צנצנת פארטי מיקס מעדני ים קראנץ</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
@@ -19890,7 +19890,7 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>12606926</t>
+          <t>12364794</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
@@ -19899,10 +19899,10 @@
         </is>
       </c>
       <c r="F365" t="n">
-        <v>10.2</v>
+        <v>50.67</v>
       </c>
       <c r="G365" t="n">
-        <v>12.04</v>
+        <v>59.79</v>
       </c>
       <c r="H365">
         <f>הגדרות!B8</f>
@@ -19933,7 +19933,7 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>דנטלייף לכלב מגזע גדול</t>
+          <t>פריסקיז צנצנת פארטי מיקס אוריגי'נל קראנץ</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -19943,7 +19943,7 @@
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>12606948</t>
+          <t>12349730</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
@@ -19952,10 +19952,10 @@
         </is>
       </c>
       <c r="F366" t="n">
-        <v>10.2</v>
+        <v>50.67</v>
       </c>
       <c r="G366" t="n">
-        <v>12.04</v>
+        <v>59.79</v>
       </c>
       <c r="H366">
         <f>הגדרות!B8</f>
@@ -19986,7 +19986,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>דנטלייף חתול עוף</t>
+          <t>דנטלייף לכלב מגזע קטן</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -19996,7 +19996,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>12607325</t>
+          <t>12606950</t>
         </is>
       </c>
       <c r="E367" t="inlineStr">
@@ -20005,10 +20005,10 @@
         </is>
       </c>
       <c r="F367" t="n">
-        <v>6.5</v>
+        <v>10.2</v>
       </c>
       <c r="G367" t="n">
-        <v>7.67</v>
+        <v>12.04</v>
       </c>
       <c r="H367">
         <f>הגדרות!B8</f>
@@ -20039,7 +20039,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>דנטלייף חתול סלמון</t>
+          <t>דנטלייף לכלב מגזע בינוני</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -20049,7 +20049,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>12607342</t>
+          <t>12606926</t>
         </is>
       </c>
       <c r="E368" t="inlineStr">
@@ -20058,10 +20058,10 @@
         </is>
       </c>
       <c r="F368" t="n">
-        <v>6.5</v>
+        <v>10.2</v>
       </c>
       <c r="G368" t="n">
-        <v>7.67</v>
+        <v>12.04</v>
       </c>
       <c r="H368">
         <f>הגדרות!B8</f>
@@ -20092,7 +20092,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>פליקס שלוקים Joyables עוף</t>
+          <t>דנטלייף לכלב מגזע גדול</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -20102,7 +20102,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>12620437</t>
+          <t>12606948</t>
         </is>
       </c>
       <c r="E369" t="inlineStr">
@@ -20111,10 +20111,10 @@
         </is>
       </c>
       <c r="F369" t="n">
-        <v>8.49</v>
+        <v>10.2</v>
       </c>
       <c r="G369" t="n">
-        <v>10.02</v>
+        <v>12.04</v>
       </c>
       <c r="H369">
         <f>הגדרות!B8</f>
@@ -20145,7 +20145,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>פליקס שלוקים Joyables סלמון</t>
+          <t>דנטלייף חתול עוף</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -20155,7 +20155,7 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>12620438</t>
+          <t>12607325</t>
         </is>
       </c>
       <c r="E370" t="inlineStr">
@@ -20164,10 +20164,10 @@
         </is>
       </c>
       <c r="F370" t="n">
-        <v>8.49</v>
+        <v>6.5</v>
       </c>
       <c r="G370" t="n">
-        <v>10.02</v>
+        <v>7.67</v>
       </c>
       <c r="H370">
         <f>הגדרות!B8</f>
@@ -20198,7 +20198,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>פליקס שלוקים Joyables ברווז</t>
+          <t>דנטלייף חתול סלמון</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -20208,7 +20208,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>12620419</t>
+          <t>12607342</t>
         </is>
       </c>
       <c r="E371" t="inlineStr">
@@ -20217,10 +20217,10 @@
         </is>
       </c>
       <c r="F371" t="n">
-        <v>8.49</v>
+        <v>6.5</v>
       </c>
       <c r="G371" t="n">
-        <v>10.02</v>
+        <v>7.67</v>
       </c>
       <c r="H371">
         <f>הגדרות!B8</f>
@@ -20251,7 +20251,7 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>פרו פלאן חטיפי DentalCare לכלב מגזע קטן</t>
+          <t>פליקס שלוקים Joyables עוף</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
@@ -20261,7 +20261,7 @@
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t>12604543</t>
+          <t>12620437</t>
         </is>
       </c>
       <c r="E372" t="inlineStr">
@@ -20270,10 +20270,10 @@
         </is>
       </c>
       <c r="F372" t="n">
-        <v>25.64</v>
+        <v>8.49</v>
       </c>
       <c r="G372" t="n">
-        <v>30.26</v>
+        <v>10.02</v>
       </c>
       <c r="H372">
         <f>הגדרות!B8</f>
@@ -20304,7 +20304,7 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>פרו פלאן חטיפי DentalCare לכלב מגזע בינוני</t>
+          <t>פליקס שלוקים Joyables סלמון</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -20314,7 +20314,7 @@
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>12604772</t>
+          <t>12620438</t>
         </is>
       </c>
       <c r="E373" t="inlineStr">
@@ -20323,10 +20323,10 @@
         </is>
       </c>
       <c r="F373" t="n">
-        <v>25.64</v>
+        <v>8.49</v>
       </c>
       <c r="G373" t="n">
-        <v>30.26</v>
+        <v>10.02</v>
       </c>
       <c r="H373">
         <f>הגדרות!B8</f>
@@ -20357,7 +20357,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>פרו פלאן חטיפי DentalCare לכלב מגזע גדול</t>
+          <t>פליקס שלוקים Joyables ברווז</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
@@ -20367,7 +20367,7 @@
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>12604733</t>
+          <t>12620419</t>
         </is>
       </c>
       <c r="E374" t="inlineStr">
@@ -20376,10 +20376,10 @@
         </is>
       </c>
       <c r="F374" t="n">
-        <v>25.64</v>
+        <v>8.49</v>
       </c>
       <c r="G374" t="n">
-        <v>30.26</v>
+        <v>10.02</v>
       </c>
       <c r="H374">
         <f>הגדרות!B8</f>
@@ -20410,7 +20410,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>דוגלי אקטיב בקר</t>
+          <t>פרו פלאן חטיפי DentalCare לכלב מגזע קטן</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -20420,7 +20420,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>12466720</t>
+          <t>12604543</t>
         </is>
       </c>
       <c r="E375" t="inlineStr">
@@ -20429,10 +20429,10 @@
         </is>
       </c>
       <c r="F375" t="n">
-        <v>114.19</v>
+        <v>25.64</v>
       </c>
       <c r="G375" t="n">
-        <v>134.74</v>
+        <v>30.26</v>
       </c>
       <c r="H375">
         <f>הגדרות!B8</f>
@@ -20463,7 +20463,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>דוגלי גורים עוף</t>
+          <t>פרו פלאן חטיפי DentalCare לכלב מגזע בינוני</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -20473,7 +20473,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>12466622</t>
+          <t>12604772</t>
         </is>
       </c>
       <c r="E376" t="inlineStr">
@@ -20482,10 +20482,10 @@
         </is>
       </c>
       <c r="F376" t="n">
-        <v>41.46</v>
+        <v>25.64</v>
       </c>
       <c r="G376" t="n">
-        <v>48.92</v>
+        <v>30.26</v>
       </c>
       <c r="H376">
         <f>הגדרות!B8</f>
@@ -20516,7 +20516,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>דוגלי גזע קטן בקר</t>
+          <t>פרו פלאן חטיפי DentalCare לכלב מגזע גדול</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
@@ -20526,7 +20526,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>12613172</t>
+          <t>12604733</t>
         </is>
       </c>
       <c r="E377" t="inlineStr">
@@ -20535,10 +20535,10 @@
         </is>
       </c>
       <c r="F377" t="n">
-        <v>39.49</v>
+        <v>25.64</v>
       </c>
       <c r="G377" t="n">
-        <v>46.6</v>
+        <v>30.26</v>
       </c>
       <c r="H377">
         <f>הגדרות!B8</f>
@@ -20569,7 +20569,7 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>דוגלי בוגר עוף</t>
+          <t>דוגלי אקטיב בקר</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
@@ -20579,7 +20579,7 @@
       </c>
       <c r="D378" t="inlineStr">
         <is>
-          <t>12368765</t>
+          <t>12466720</t>
         </is>
       </c>
       <c r="E378" t="inlineStr">
@@ -20588,10 +20588,10 @@
         </is>
       </c>
       <c r="F378" t="n">
-        <v>37.61</v>
+        <v>114.19</v>
       </c>
       <c r="G378" t="n">
-        <v>44.38</v>
+        <v>134.74</v>
       </c>
       <c r="H378">
         <f>הגדרות!B8</f>
@@ -20622,7 +20622,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>דוגלי בוגר בקר</t>
+          <t>דוגלי גורים עוף</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
@@ -20632,7 +20632,7 @@
       </c>
       <c r="D379" t="inlineStr">
         <is>
-          <t>12368766</t>
+          <t>12466622</t>
         </is>
       </c>
       <c r="E379" t="inlineStr">
@@ -20641,10 +20641,10 @@
         </is>
       </c>
       <c r="F379" t="n">
-        <v>37.61</v>
+        <v>41.46</v>
       </c>
       <c r="G379" t="n">
-        <v>44.38</v>
+        <v>48.92</v>
       </c>
       <c r="H379">
         <f>הגדרות!B8</f>
@@ -20675,7 +20675,7 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>דוגלי בוגר עוף</t>
+          <t>דוגלי גזע קטן בקר</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
@@ -20685,7 +20685,7 @@
       </c>
       <c r="D380" t="inlineStr">
         <is>
-          <t>12368676</t>
+          <t>12613172</t>
         </is>
       </c>
       <c r="E380" t="inlineStr">
@@ -20694,10 +20694,10 @@
         </is>
       </c>
       <c r="F380" t="n">
-        <v>108.76</v>
+        <v>39.49</v>
       </c>
       <c r="G380" t="n">
-        <v>128.34</v>
+        <v>46.6</v>
       </c>
       <c r="H380">
         <f>הגדרות!B8</f>
@@ -20728,7 +20728,7 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>דוגלי בוגר בקר</t>
+          <t>דוגלי בוגר עוף</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
@@ -20738,7 +20738,7 @@
       </c>
       <c r="D381" t="inlineStr">
         <is>
-          <t>12368675</t>
+          <t>12368765</t>
         </is>
       </c>
       <c r="E381" t="inlineStr">
@@ -20747,10 +20747,10 @@
         </is>
       </c>
       <c r="F381" t="n">
-        <v>108.76</v>
+        <v>37.61</v>
       </c>
       <c r="G381" t="n">
-        <v>128.34</v>
+        <v>44.38</v>
       </c>
       <c r="H381">
         <f>הגדרות!B8</f>
@@ -20770,6 +20770,165 @@
       </c>
       <c r="L381">
         <f>I381*(1+J381/100)+K381</f>
+        <v/>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>פורינה (חנויות)</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>דוגלי בוגר בקר</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>חטיפים</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>12368766</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="F382" t="n">
+        <v>37.61</v>
+      </c>
+      <c r="G382" t="n">
+        <v>44.38</v>
+      </c>
+      <c r="H382">
+        <f>הגדרות!B8</f>
+        <v/>
+      </c>
+      <c r="I382">
+        <f>F382*(1-H382/100)*1.18</f>
+        <v/>
+      </c>
+      <c r="J382">
+        <f>הגדרות!C8</f>
+        <v/>
+      </c>
+      <c r="K382">
+        <f>הגדרות!D8</f>
+        <v/>
+      </c>
+      <c r="L382">
+        <f>I382*(1+J382/100)+K382</f>
+        <v/>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>פורינה (חנויות)</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>דוגלי בוגר עוף</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>חטיפים</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>12368676</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="F383" t="n">
+        <v>108.76</v>
+      </c>
+      <c r="G383" t="n">
+        <v>128.34</v>
+      </c>
+      <c r="H383">
+        <f>הגדרות!B8</f>
+        <v/>
+      </c>
+      <c r="I383">
+        <f>F383*(1-H383/100)*1.18</f>
+        <v/>
+      </c>
+      <c r="J383">
+        <f>הגדרות!C8</f>
+        <v/>
+      </c>
+      <c r="K383">
+        <f>הגדרות!D8</f>
+        <v/>
+      </c>
+      <c r="L383">
+        <f>I383*(1+J383/100)+K383</f>
+        <v/>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>פורינה (חנויות)</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>דוגלי בוגר בקר</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>חטיפים</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>12368675</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="F384" t="n">
+        <v>108.76</v>
+      </c>
+      <c r="G384" t="n">
+        <v>128.34</v>
+      </c>
+      <c r="H384">
+        <f>הגדרות!B8</f>
+        <v/>
+      </c>
+      <c r="I384">
+        <f>F384*(1-H384/100)*1.18</f>
+        <v/>
+      </c>
+      <c r="J384">
+        <f>הגדרות!C8</f>
+        <v/>
+      </c>
+      <c r="K384">
+        <f>הגדרות!D8</f>
+        <v/>
+      </c>
+      <c r="L384">
+        <f>I384*(1+J384/100)+K384</f>
         <v/>
       </c>
     </row>

</xml_diff>